<commit_message>
12th Commit : Browser Size Adjusted In ABCD Hybrid Framework
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76EC1EA8-2C6E-4EC3-94A5-E0208F982DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7F49A6-7881-4CCD-BC27-6A3F8FECECAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -3116,12 +3116,49 @@
 4.Click Login,click,,"//button[@type='submit']"
 5.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
 6.Load User App,switch_to,user,
-7.wait,5000,,
-8.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-9.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-9.wait,3000,,
-10.Load Driver App,switch_to,driver,
-11.wait,5000,,
+7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+11.wait,1000,,
+12.Load Driver App,switch_to,driver,
+13.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
+14.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
+15.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
+16.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
+17.wait,1000,,
+18.Load  Super Admn,switch_to,web,
+19.wait,1000,,
+20. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+21.Click City area menu,click,,"//span[normalize-space()='City Area']"
+22.Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
+23.Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
+24.Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
+25.Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
+26.Open Status Dropdown,click,,"//span[@aria-label='select status']"
+27.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
+28.Enter City Area, type, triplicane, "//input[@placeholder='Search location']"
+29.wait,1000,,
+30.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
+31.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
+32.wait,1000,,
+33. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
+34. Click Submit,click,,"//button[normalize-space()='Submit']"
+35. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
+36. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
+37. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
+38. Click Add Category,click,,"//button[normalize-space()='Add Category']"
+39. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
+40. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
+41. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
+42. Click close,click,,"//button[normalize-space()='Close']"
+43. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
+44. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
+45. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
+46.Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
+47. Open Select City Dropdown,click,,"//select[@id='cityId']"
+48. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
+49. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
 </t>
   </si>
 </sst>
@@ -4253,7 +4290,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="259.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>108</v>
       </c>

</xml_diff>

<commit_message>
16th Commit : Hybrid Regression Test Sutite Added
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,29 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7F49A6-7881-4CCD-BC27-6A3F8FECECAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C04DED92-5AA5-4ED7-8740-52D855B120B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="14" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
-    <sheet name="UniversalFlow" sheetId="31" r:id="rId2"/>
-    <sheet name="AddCustomer" sheetId="13" r:id="rId3"/>
-    <sheet name="AddCityArea" sheetId="1" r:id="rId4"/>
-    <sheet name="AddCityAdmin" sheetId="2" r:id="rId5"/>
-    <sheet name="AddAutoDriver" sheetId="3" r:id="rId6"/>
-    <sheet name="AddBikeDriver" sheetId="4" r:id="rId7"/>
-    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId8"/>
-    <sheet name="TransportServiceCompleteTest" sheetId="15" r:id="rId9"/>
-    <sheet name="AddStore" sheetId="7" r:id="rId10"/>
-    <sheet name="StoreOperations" sheetId="8" r:id="rId11"/>
-    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId12"/>
-    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId13"/>
-    <sheet name="AddProvider" sheetId="11" r:id="rId14"/>
-    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId15"/>
-    <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId16"/>
-    <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId17"/>
-    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId18"/>
+    <sheet name="AddCustomer" sheetId="13" r:id="rId2"/>
+    <sheet name="AddCityArea" sheetId="1" r:id="rId3"/>
+    <sheet name="AddCityAdmin" sheetId="2" r:id="rId4"/>
+    <sheet name="AddAutoDriver" sheetId="3" r:id="rId5"/>
+    <sheet name="AddBikeDriver" sheetId="4" r:id="rId6"/>
+    <sheet name="AddTaxiDriver" sheetId="5" r:id="rId7"/>
+    <sheet name="TransportServiceCompleteTest" sheetId="15" r:id="rId8"/>
+    <sheet name="AddStore" sheetId="7" r:id="rId9"/>
+    <sheet name="StoreOperations" sheetId="8" r:id="rId10"/>
+    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId11"/>
+    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId12"/>
+    <sheet name="AddProvider" sheetId="11" r:id="rId13"/>
+    <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId14"/>
+    <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId15"/>
+    <sheet name="AddTransportCityAdmin" sheetId="30" r:id="rId16"/>
+    <sheet name="DataCleanUpSheet" sheetId="28" r:id="rId17"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="108">
   <si>
     <t>City Area</t>
   </si>
@@ -3096,70 +3095,6 @@
 176.Click  Submit,click,,"//button[normalize-space()='Submit']"
 177.Verify Sucess, verify, , "//div[@aria-label='Info']"
 178.wait,2000,,</t>
-  </si>
-  <si>
-    <t>SA_TS_33</t>
-  </si>
-  <si>
-    <t>UniversalFlow</t>
-  </si>
-  <si>
-    <t>TC_CA_00_Universal_Flow</t>
-  </si>
-  <si>
-    <t>UniversalFlow is verified</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.Load Site,navigate,https://dev.we1.co/#/login,
-2.Enter  Email , type , super_admin@gmail.com, "//input[@placeholder='Enter your email']"
-3.Enter Password,type,R1mep@321, "//input[@placeholder='Enter your password']"
-4.Click Login,click,,"//button[@type='submit']"
-5.Verify Dashboard,verify,,"//div[contains(text(),'Date Wise Statistics')]"
-6.Load User App,switch_to,user,
-7.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-8.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-9.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-10.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-11.wait,1000,,
-12.Load Driver App,switch_to,driver,
-13.Click English  Icon,tap,,"//android.widget.Button[@content-desc="English"]"
-14.Click Next,tap,,"//android.widget.Button[@content-desc="Next"]"
-15.Click Mobile Number,tap,,"//android.widget.Button[@content-desc="Mobile Number"]"
-16.Click Close,tap,,"//android.widget.ImageView[@content-desc="Cancel"]"
-17.wait,1000,,
-18.Load  Super Admn,switch_to,web,
-19.wait,1000,,
-20. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-21.Click City area menu,click,,"//span[normalize-space()='City Area']"
-22.Verify City Area List,verify,,"//div[contains(text(),'City Area List')]"
-23.Click Add City Area button , click ,, "//button[contains(@class, 'buttonWidget') and contains(text(), 'Add City Area')]"
-24.Verify City Area heading,verify,,"//div[contains(text(), 'City Area') and contains(@style, 'font-weight: 700')]"
-25.Enter Area Name, type, triplicane_{timestamp} &gt;&gt; areaName, "//input[@placeholder='Area Name']"
-26.Open Status Dropdown,click,,"//span[@aria-label='select status']"
-27.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-28.Enter City Area, type, triplicane, "//input[@placeholder='Search location']"
-29.wait,1000,,
-30.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-31.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-32.wait,1000,,
-33. draw polygon, "-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120", //div[@class='ol-layer']//canvas
-34. Click Submit,click,,"//button[normalize-space()='Submit']"
-35. Verify Success Message,verify,,"//div[@aria-label='Added Successfully']"
-36. Click Transport Services,click,,"//div[.//h2[normalize-space()='Transport Services']]"
-37. Verify Transport Page,verify,,"//div[contains(text(),'TRANSPORT SERVICES')]"
-38. Click Add Category,click,,"//button[normalize-space()='Add Category']"
-39. Open Select City Dropdown,click,,"//div[@class='p-element p-multiselect-label-container']"
-40. Search City Area,type,{areaName},"//input[contains(@class,'p-multiselect-filter')]"
-41. Verify Area in Dropdown,verify,,"//li[@role='option'][contains(.,'{areaName}')]"
-42. Click close,click,,"//button[normalize-space()='Close']"
-43. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-44. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-45. Verify City Admin List,verify,,"//div[contains(text(),'City Admin List')]"
-46.Click Add City Admin button , click ,, "//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-47. Open Select City Dropdown,click,,"//select[@id='cityId']"
-48. Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-49. Verify Selection,verify,,"//select[@id='cityId'][contains(.,'{areaName}')]"
-</t>
   </si>
 </sst>
 </file>
@@ -3607,78 +3542,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="24" customWidth="1"/>
-    <col min="3" max="3" width="26.77734375" customWidth="1"/>
-    <col min="4" max="4" width="34.109375" customWidth="1"/>
-    <col min="5" max="5" width="69.33203125" customWidth="1"/>
-    <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="8"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3750,7 +3613,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3822,7 +3685,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73960651-1493-478A-BEDA-A31CF297E315}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3894,7 +3757,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F63FB6C5-854C-4D7D-9CEB-846B4D7D2F52}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3966,7 +3829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ADEF0-2336-4246-BBC3-461C4994D500}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4038,7 +3901,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0F6277B-DBCF-4BFF-819C-1E90748D3258}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4110,7 +3973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6B7FC7-76CD-491F-AC51-1837B3B068AC}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4175,7 +4038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F2F621F-9A1F-4BCF-BC43-4FD25385804C}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4250,82 +4113,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1717BC20-9348-4B52-9588-34F52BC8B75D}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="4" max="4" width="26.6640625" customWidth="1"/>
-    <col min="5" max="5" width="53.21875" customWidth="1"/>
-    <col min="6" max="6" width="36.88671875" customWidth="1"/>
-    <col min="7" max="7" width="16.33203125" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ECEE02-404F-4AF1-8311-95653C3B218B}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4401,7 +4188,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4477,7 +4264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9466ABF-463D-46B5-A321-4AC4765F1CE7}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4542,7 +4329,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7A75689-8D07-4A99-AA90-48806EECB90F}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4614,7 +4401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4197A722-266E-4219-9B46-8F4D56D7D7A1}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4686,7 +4473,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{790BFFF3-3BE5-4068-A6FF-6214BEDD72BA}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4758,7 +4545,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4DB4E5D-EBF5-4B6A-BF83-7934D70C5535}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4829,4 +4616,76 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="26.77734375" customWidth="1"/>
+    <col min="4" max="4" width="34.109375" customWidth="1"/>
+    <col min="5" max="5" width="69.33203125" customWidth="1"/>
+    <col min="6" max="6" width="31.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
62th Commit : Customer Locator Implemented Crashproof
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3ACB132-3CED-47AB-9032-CAFCB3B4D90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCF66921-EDF0-49EC-BE24-DF4079088636}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -3027,7 +3027,7 @@
 10.Upload Profile Image, uploadfile, "src/main/resources/test-data/customer.jpg", "admin.customer.upload_profile_img"
 11.Click Submit, click, , "admin.customer.submit_btn"
 12.Verify Added Succesfully, verify, , "admin.customer.toast_info"
-13. Click Customer Icon,click,,"admin.menu.customer_icon"
+13. Click Dashboard,click,,"admin.menu.dashboard"
 14. Click Customer Icon,click,,"admin.menu.customer_icon"
 15.Click Verified Customers,click,,"admin.menu.verified_customers"
 16. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
@@ -3048,7 +3048,7 @@
 31.Select Deduct Money,click,,"admin.customer.wallet.select_deduct_money"
 32.Click Submit, click, , "admin.customer.submit_btn"
 33.Verify Saved Succesfully, verify, , "admin.customer.toast_added_success"
-34. Click Customer Icon,click,,"admin.menu.customer_icon"
+34. Click dashbaord Icon,click,,"admin.menu.dashboard"
 35. Click Customer Icon,click,,"admin.menu.customer_icon"
 36.Click Verified Customers,click,,"admin.menu.verified_customers"
 37. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
@@ -3071,7 +3071,7 @@
 54.Enter Points, type, 10, "admin.customer.loyalty.input_points"
 55.Click Submit, click, , "admin.customer.submit_btn"
 56.Verify Added Succesfully, verify, , "admin.customer.toast_info"
-57. Click Customer Icon,click,,"admin.menu.customer_icon"
+57. Click Dashboard Icon,click,,"admin.menu.dashboard"
 58. Click Customer Icon,click,,"admin.menu.customer_icon"
 59.Click Verified Customers,click,,"admin.menu.verified_customers"
 60. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
@@ -3082,14 +3082,14 @@
 65.Disable Reason,type,Client Complaints,"admin.customer.dialog.textarea_reason"
 66.Click Reject Yes,click,,"admin.customer.dialog.btn_confirm_yes"
 67.Verify Added Succesfully, verify, , "admin.customer.toast_info"
-68. Click Customer Icon,click,,"admin.menu.customer_icon"
+68. Click Dashboard Icon,click,,"admin.menu.dashboard"
 69. Click Customer Icon,click,,"admin.menu.customer_icon"
 70.Click Blocked Customers,click,,"admin.menu.blocked_customers"
 71.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
 72.Scroll Grid, tab, 10, "admin.customer.filter_name"
 73.Click Enable Icon,click,,"admin.customer.grid.btn_status_enable"
 74.Click Enable Yes,click,,"admin.customer.dialog.btn_confirm_yes"
-75. Click Customer Icon,click,,"admin.menu.customer_icon"
+75. Click Dashboard Icon,click,,"admin.menu.dashboard"
 76. Click Customer Icon,click,,"admin.menu.customer_icon"
 77.Click Verified Customers,click,,"admin.menu.verified_customers"
 78. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"

</xml_diff>

<commit_message>
66th Commit : City Admin Locator Implemented
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B60783-E1EF-4901-A479-BBF4161F3A04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5DFE3E-5BF2-403F-A2BB-AD8A965689B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
     <sheet name="AddCustomer" sheetId="31" r:id="rId2"/>
     <sheet name="AddCityArea" sheetId="1" r:id="rId3"/>
-    <sheet name="AddCityAdmin" sheetId="2" r:id="rId4"/>
+    <sheet name="AddCityAdmin" sheetId="32" r:id="rId4"/>
     <sheet name="AddAutoDriver" sheetId="3" r:id="rId5"/>
     <sheet name="AddBikeDriver" sheetId="4" r:id="rId6"/>
     <sheet name="AddTaxiDriver" sheetId="5" r:id="rId7"/>
@@ -2930,145 +2930,18 @@
 178.wait,2000,,</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-2. Click Setting menu,click,,"//i[contains(@class,'fa-cog')]"
-3. Click City admin menu,click,,"//span[normalize-space()='City Admin']"
-4. Verify City Admin List,verify,,"//div[normalize-space()='City Admin List']"
-5. Click Add City Admin button,click,,"//button[contains(@class, 'buttonWidget') and normalize-space()='Add City Admin']"
-6. Verify City Admin heading,verify,,"//h2[@class='text-base font-semibold text-gray-800']"
-7.Select Name field,click ,, "//input[@id='name']"
-8. Enter Admin Name, type, faizal{randomAlpha} &gt;&gt; adminName, "//input[@id='name']"
-9.Select Email field,click,, "//input[@id='email']"
-10. Enter Email, type, faizal_{timestamp}@gmail.com, "//input[@id='email']"
-11.select the password field,click,, "//input[@id='password']"
-12.Enter the Password as "faizal@123". "//input[@id='password']"
-13.Open Select City Dropdown,click,,"//select[@id='cityId']"
-14.Select {areaName},click,,"//option[contains(text(),'{areaName}')][last()]"
-15. Click on the "Transport Service" → "Auto Ride" checkbox. "//label[normalize-space()='Auto Ride']"
-16.Click on the "Customers" → "Add Customers" checkbox. "//label[normalize-space()='Add Customers']"
-17.Click on the "Customers" → "Verified Customers"checkbox. "//label[normalize-space()='Verified Customers']"
-18.Click on the "Customers" → "Non Verified Customers" checkbox. "//label[normalize-space()='Non Verified Customers']"
-19.Click on the "Customers" → "Blocked Customers" checkbox. "//label[normalize-space()='Blocked Customers']"
-20.Click on the "Customers" → "Deleted Customers" checkbox. "//label[normalize-space()='Deleted Customers']"
-21.Click on the "Customers" → "Pending Customers" checkbox. "//label[normalize-space()='Pending Customers']"
-22.Click on the "Providers" → "Transport Providers List" checkbox. "//label[normalize-space()='Transport Providers List']"
-23.Click on the "Drivers" → "Add Driver" checkbox."//label[normalize-space()='Add Driver']"
-24.Click on the "Drivers" → "Approved Drivers" checkbox. "//label[normalize-space()='Approved Drivers']"
-25.Click on the "Drivers" → "Un-Approved Drivers" checkbox. "//label[normalize-space()='Un-Approved Drivers']"
-26.Click on the "Drivers" → "Blocked Drivers" checkbox. "//label[normalize-space()='Blocked Drivers']"
-27.Click on the "Drivers" → "Reject Drivers" checkbox. "//label[normalize-space()='Reject Drivers']"
-28.Click on the "Drivers" → "Deleted Drivers" checkbox. "//label[normalize-space()='Deleted Drivers']"
-29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox. "//label[normalize-space()='Driver Subscription Plan']"
-30.Click on the "Cash Out" → "Driver Cash Out" checkbox. "//label[normalize-space()='Driver Cash Out']"
-31.Click on the "Report Issue" → "Customer Report Issues" checkbox. "//label[normalize-space()='Customer Report Issues']"
-32.Click on the "Report Issue" → "Driver Report Issues" checkbox. "//label[normalize-space()='Driver Report Issues']"
-33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,"//label[normalize-space()='Provider Report Issues']"
-34.Click on the "Report Issue" → "Report issue settings" checkbox. "//label[normalize-space()='Report issue settings']"
-35.Click on the "Report Issue" → "FAQs" checkbox. "(//h3[contains(.,'Report Issue')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox. "//label[normalize-space()='Header &amp; Footer']"
-37.Click on the "Website Settings" → "Home Page Settings" checkbox. "//label[normalize-space()='Home Page']"
-38.Click on the "Website Settings" → "Delivery Settings" checkbox. "//div[h3[contains(.,'Website Settings')]]//label[contains(.,'Delivery')]"
-39.Click on the "Website Settings" → "Transport Settings" checkbox. "//div[.//h3[contains(text(),'Website Settings')]]//label[contains(.,'Transport')]"
-40.Click on the "Website Settings" → "FAQs" checkbox. "(//h3[contains(.,'Website Settings')]/following-sibling::div//label[contains(.,'FAQs')])[1]"
-41.Click Submit,click,,"//button[@type='submit']"
-42. Verify Success Message,verify,,"//div[@aria-label='Info']"
-43.Filter admin name,type,{adminName},"//input[@aria-label='Name Filter Input']"
-</t>
-  </si>
-  <si>
     <t>1. Enter  Email , type , super_admin@gmail.com, "web.global.login.email"
 2. Enter Password,type,R1mep@321, "web.global.login.password"
 3. Click Login,click,,"web.global.login.submit_btn"
-4. Verify Dashboard,verify,,"web.global.dashboard.statistics_header"</t>
-  </si>
-  <si>
-    <t>1. Click Customer Icon,click,,"admin.menu.customer_icon"
-2. Click Add Customers,click,,"admin.menu.add_customers"
-3. Verify Add Customer Heading,verify,,"admin.customer.add_heading"
-4. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
-5. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
-6. Enter Contact Number,type,{randomPhone},"admin.customer.input_phone"
-7. Enter Video Call Limit,type,60,"admin.customer.input_video_limit"
-8. Open Gender,click,,"admin.customer.dropdown_gender"
-9. Select Male,click,,"admin.customer.select_gender_male"
-10. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
-11. Click Submit,click,,"web.global.action.submit"
-12. Verify Added Successfully,verify,,"web.global.toast.info"
-13. Click Dashboard,click,,"web.global.menu.dashboard"
-14. Click Customer Icon,click,,"admin.menu.customer_icon"
-15. Click Verified Customers,click,,"admin.menu.verified_customers"
-16. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
-17. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
-18. Scroll Grid,tab,7,"admin.customer.filter_name"
-19. Click Edit Icon,click,,"admin.customer.grid.btn_edit"
-20. Click Close,click,,"web.global.action.close"
-21. Click Wallet Icon,click,,"admin.customer.grid.btn_wallet"
-22. Click Add Money,click,,"admin.customer.wallet.btn_add_money"
-23. Enter Wallet Amount,type,1000,"admin.customer.wallet.input_amount"
-24. Open Choose Option Dropdown,click,,"admin.customer.wallet.dropdown_option"
-25. Select Add Money,click,,"admin.customer.wallet.select_add_money"
-26. Click Submit,click,,"web.global.action.submit"
-27. Verify Saved Successfully,verify,,"web.global.toast.success"
-28. Click Add Money,click,,"admin.customer.wallet.btn_add_money"
-29. Enter Wallet Amount,type,200,"admin.customer.wallet.input_amount"
-30. Open Choose Option Dropdown,click,,"admin.customer.wallet.dropdown_option"
-31. Select Deduct Money,click,,"admin.customer.wallet.select_deduct_money"
-32. Click Submit,click,,"web.global.action.submit"
-33. Verify Saved Successfully,verify,,"web.global.toast.success"
-34. Click dashboard Icon,click,,"web.global.menu.dashboard"
-35. Click Customer Icon,click,,"admin.menu.customer_icon"
-36. Click Verified Customers,click,,"admin.menu.verified_customers"
-37. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
-38. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
-39. Scroll Grid,tab,7,"admin.customer.filter_name"
-40. Click Loyalty Points Icon,click,,"admin.customer.grid.btn_loyalty_points"
-41. Click Manage Loyalty Points,click,,"admin.customer.loyalty.btn_manage"
-42. Open Service Dropdown,click,,"admin.customer.loyalty.dropdown_service"
-43. Select Bike Ride,click,,"admin.customer.loyalty.select_bike_ride"
-44. Open Choose Option Dropdown,click,,"admin.customer.loyalty.dropdown_option"
-45. Select Add Points,click,,"admin.customer.loyalty.select_add_points"
-46. Enter Points,type,30,"admin.customer.loyalty.input_points"
-47. Click Submit,click,,"web.global.action.submit"
-48. Verify Added Successfully,verify,,"web.global.toast.info"
-49. Click Manage Loyalty Points,click,,"admin.customer.loyalty.btn_manage"
-50. Open Service Dropdown,click,,"admin.customer.loyalty.dropdown_service"
-51. Select Bike Ride,click,,"admin.customer.loyalty.select_bike_ride"
-52. Open Choose Option Dropdown,click,,"admin.customer.loyalty.dropdown_option"
-53. Select Deduct Points,click,,"admin.customer.loyalty.select_deduct_points"
-54. Enter Points,type,10,"admin.customer.loyalty.input_points"
-55. Click Submit,click,,"web.global.action.submit"
-56. Verify Added Successfully,verify,,"web.global.toast.info"
-57. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-58. Click Customer Icon,click,,"admin.menu.customer_icon"
-59. Click Verified Customers,click,,"admin.menu.verified_customers"
-60. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
-61. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
-62. Scroll Grid,tab,7,"admin.customer.filter_name"
-63. Click Disable Icon,click,,"admin.customer.grid.btn_block"
-64. Click Disable User Yes,click,,"web.global.dialog.btn_confirm_yes"
-65. Disable Reason,type,Client Complaints,"web.global.dialog.textarea_reason"
-66. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
-67. Verify Added Successfully,verify,,"web.global.toast.info"
-68. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-69. Click Customer Icon,click,,"admin.menu.customer_icon"
-70. Click Blocked Customers,click,,"admin.menu.blocked_customers"
-71. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
-72. Scroll Grid,tab,10,"admin.customer.filter_name"
-73. Click Enable Icon,click,,"admin.customer.grid.btn_status_enable"
-74. Click Enable Yes,click,,"web.global.dialog.btn_confirm_yes"
-75. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-76. Click Customer Icon,click,,"admin.menu.customer_icon"
-77. Click Verified Customers,click,,"admin.menu.verified_customers"
-78. Verify Verified Customer List Heading,verify,,"admin.customer.verified_list_heading"
-79. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
+4.Load Dashboard,wait_until_visible,,"web.global.dashboard.statistics_header"</t>
   </si>
   <si>
     <t xml:space="preserve">1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
 2. Click Setting menu,click,,"web.global.menu.settings"
 3. Click City area menu,click,,"admin.menu.city_area"
-4. Verify City Area List,verify,,"admin.city_area.list_heading"
+4. Wait For Area List,wait_until_visible,,"admin.city_area.list_heading"
 5. Click Add City Area button,click,,"admin.city_area.btn_add"
-6. Verify City Area heading,verify,,"admin.city_area.add_heading"
+6. Wait For City Area heading,wait_until_visible,,"admin.city_area.add_heading"
 7. Enter Area Name,type,triplicane_{timestamp} &gt;&gt; areaName,"admin.city_area.input_name"
 8. Open Status Dropdown,click,,"admin.city_area.dropdown_status"
 9. Select Active,click,,"admin.city_area.select_status_active"
@@ -3079,22 +2952,151 @@
 14. wait,1000,,
 15. Map Polygon,draw polygon,"-120;-120 : 120;-120 : 120;120 : -120;120 : -120;-120","//div[@class='ol-layer']//canvas"
 16. Click Submit,click,,"web.global.action.submit"
-17. Verify Success Message,verify,,"web.global.toast.success"
+17. Wait For Success Message,wait_until_visible,,"web.global.toast.success"
 18. Click Transport Services,click,,"admin.transport.card_link"
-19. Verify Transport Page,verify,,"admin.transport.page_heading"
+19. Wait For Transport Page,wait_until_visible,,"admin.transport.page_heading"
 20. Click Add Category,click,,"admin.transport.btn_add_category"
 21. Open Select City Dropdown,click,,"admin.transport.dropdown_city_multiselect"
 22. Search City Area,type,{areaName},"admin.transport.input_filter_city"
 23. Verify Area in Dropdown,verify,,"admin.transport.select_filtered_option"
 24. Click close,click,,"web.global.action.close"
-25. Click Setting menu,click,,"web.global.menu.settings"
-26. Click City admin menu,click,,"admin.menu.city_admin"
-27. Verify City Admin List,verify,,"admin.city_admin.list_heading"
-28. Click Add City Admin button,click,,"admin.city_admin.btn_add"
-29. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
-30. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
-31. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
+25.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+26. Click Setting menu,click,,"web.global.menu.settings"
+27. Click City admin menu,click,,"admin.menu.city_admin"
+28. Wait For City Admin List,wait_until_visible,,"admin.city_admin.list_heading"
+29. Click Add City Admin button,click,,"admin.city_admin.btn_add"
+30. Open Select City Dropdown,click,,"admin.city_admin.select_city_dropdown"
+31. Select {areaName},click,,"admin.city_admin.select_dynamic_option"
+32. Verify Selection,verify,,"admin.city_admin.verify_dropdown_value"
 </t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Setting menu,click,,web.global.menu.settings
+3. Click City admin menu,click,,admin.menu.city_admin
+4. Wait For City Admin List,wait_until_visible,,admin.city_admin.list_heading
+5. Click Add City Admin button,click,,admin.city_admin.btn_add
+6. Wait For Admin heading,wait_until_visible,,admin.city_admin.add_heading
+7.Select Name field,click,,admin.city_admin.input_name
+8. Enter Admin Name,type,faizal{randomAlpha} &gt;&gt; adminName,admin.city_admin.input_name
+9.Select Email field,click,,admin.city_admin.input_email
+10. Enter Email,type,faizal_{timestamp}@gmail.com,admin.city_admin.input_email
+11.select the password field,click,,admin.city_admin.input_password
+12.Enter the Password as "faizal@123",type,faizal@123,admin.city_admin.input_password
+13.Open Select City Dropdown,click,,admin.city_admin.select_city_dropdown
+14.Select {areaName},click,,admin.city_admin.select_dynamic_option
+15. Click on the "Transport Service" → "Auto Ride" checkbox,click,,admin.city_admin.chk_transport_autoride
+16.Click on the "Customers" → "Add Customers" checkbox,click,,admin.city_admin.chk_customer_add
+17.Click on the "Customers" → "Verified Customers"checkbox,click,,admin.city_admin.chk_customer_verified
+18.Click on the "Customers" → "Non Verified Customers" checkbox,click,,admin.city_admin.chk_customer_unverified
+19.Click on the "Customers" → "Blocked Customers" checkbox,click,,admin.city_admin.chk_customer_blocked
+20.Click on the "Customers" → "Deleted Customers" checkbox,click,,admin.city_admin.chk_customer_deleted
+21.Click on the "Customers" → "Pending Customers" checkbox,click,,admin.city_admin.chk_customer_pending
+22.Click on the "Providers" → "Transport Providers List" checkbox,click,,admin.city_admin.chk_provider_list
+23.Click on the "Drivers" → "Add Driver" checkbox,click,,admin.city_admin.chk_driver_add
+24.Click on the "Drivers" → "Approved Drivers" checkbox,click,,admin.city_admin.chk_driver_approved
+25.Click on the "Drivers" → "Un-Approved Drivers" checkbox,click,,admin.city_admin.chk_driver_unapproved
+26.Click on the "Drivers" → "Blocked Drivers" checkbox,click,,admin.city_admin.chk_driver_blocked
+27.Click on the "Drivers" → "Reject Drivers" checkbox,click,,admin.city_admin.chk_driver_rejected
+28.Click on the "Drivers" → "Deleted Drivers" checkbox,click,,admin.city_admin.chk_driver_deleted
+29.Click on the "Subscription Plan" → "Driver Subscription Plan" checkbox,click,,admin.city_admin.chk_subscription_plan
+30.Click on the "Cash Out" → "Driver Cash Out" checkbox,click,,admin.city_admin.chk_cashout
+31.Click on the "Report Issue" → "Customer Report Issues" checkbox,click,,admin.city_admin.chk_report_customer
+32.Click on the "Report Issue" → "Driver Report Issues" checkbox,click,,admin.city_admin.chk_report_driver
+33.Click on the "Report Issue" → "Provider Report Issues" checkbox,click,,admin.city_admin.chk_report_provider
+34.Click on the "Report Issue" → "Report issue settings" checkbox,click,,admin.city_admin.chk_report_settings
+35.Click on the "Report Issue" → "FAQs" checkbox,click,,admin.city_admin.chk_report_faqs
+36.Click on the "Website Settings" → "Header &amp; Footer Settings" checkbox,click,,admin.city_admin.chk_web_header_footer
+37.Click on the "Website Settings" → "Home Page Settings" checkbox,click,,admin.city_admin.chk_web_homepage
+38.Click on the "Website Settings" → "Delivery Settings" checkbox,click,,admin.city_admin.chk_web_delivery
+39.Click on the "Website Settings" → "Transport Settings" checkbox,click,,admin.city_admin.chk_web_transport
+40.Click on the "Website Settings" → "FAQs" checkbox,click,,admin.city_admin.chk_web_faqs
+41.Click Submit,click,,web.global.login.submit_btn
+42. Wait For Success Message,wait_until_visible,,web.global.toast.info
+43.Filter admin name,type,{adminName},admin.city_admin.input_name_filter</t>
+  </si>
+  <si>
+    <t>1. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+2. Click Customer Icon,click,,"admin.menu.customer_icon"
+3. Click Add Customers,click,,"admin.menu.add_customers"
+4. Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
+5. Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
+6. Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+7. Enter Contact Number,type,{randomPhone},"admin.customer.input_phone"
+8. Enter Video Call Limit,type,60,"admin.customer.input_video_limit"
+9. Open Gender,click,,"admin.customer.dropdown_gender"
+10. Select Male,click,,"admin.customer.select_gender_male"
+11. Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+12. Click Submit,click,,"web.global.action.submit"
+13. Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+14. Click Dashboard,click,,"web.global.menu.dashboard"
+15. Click Customer Icon,click,,"admin.menu.customer_icon"
+16. Click Verified Customers,click,,"admin.menu.verified_customers"
+17. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+18. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+19. Scroll Grid,tab,7,"admin.customer.filter_name"
+20. Click Edit Icon,click,,"admin.customer.grid.btn_edit"
+21. Click Close,click,,"web.global.action.close"
+22. Click Wallet Icon,click,,"admin.customer.grid.btn_wallet"
+23. Click Add Money,click,,"admin.customer.wallet.btn_add_money"
+24. Enter Wallet Amount,type,1000,"admin.customer.wallet.input_amount"
+25. Open Choose Option Dropdown,click,,"admin.customer.wallet.dropdown_option"
+26. Select Add Money,click,,"admin.customer.wallet.select_add_money"
+27. Click Submit,click,,"web.global.action.submit"
+28. Wait For Saved Successfully,wait_until_visible,,"web.global.toast.success"
+29. Click Add Money,click,,"admin.customer.wallet.btn_add_money"
+30. Enter Wallet Amount,type,200,"admin.customer.wallet.input_amount"
+31. Open Choose Option Dropdown,click,,"admin.customer.wallet.dropdown_option"
+32. Select Deduct Money,click,,"admin.customer.wallet.select_deduct_money"
+33. Click Submit,click,,"web.global.action.submit"
+34. Wait For Saved Successfully,wait_until_visible,,"web.global.toast.success"
+35. Click dashboard Icon,click,,"web.global.menu.dashboard"
+36. Click Customer Icon,click,,"admin.menu.customer_icon"
+37. Click Verified Customers,click,,"admin.menu.verified_customers"
+38. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+39. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+40. Scroll Grid,tab,7,"admin.customer.filter_name"
+41. Click Loyalty Points Icon,click,,"admin.customer.grid.btn_loyalty_points"
+42. Click Manage Loyalty Points,click,,"admin.customer.loyalty.btn_manage"
+43. Open Service Dropdown,click,,"admin.customer.loyalty.dropdown_service"
+44. Select Bike Ride,click,,"admin.customer.loyalty.select_bike_ride"
+45. Open Choose Option Dropdown,click,,"admin.customer.loyalty.dropdown_option"
+46. Select Add Points,click,,"admin.customer.loyalty.select_add_points"
+47. Enter Points,type,30,"admin.customer.loyalty.input_points"
+48. Click Submit,click,,"web.global.action.submit"
+49. Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+50. Click Manage Loyalty Points,click,,"admin.customer.loyalty.btn_manage"
+51. Open Service Dropdown,click,,"admin.customer.loyalty.dropdown_service"
+52. Select Bike Ride,click,,"admin.customer.loyalty.select_bike_ride"
+53. Open Choose Option Dropdown,click,,"admin.customer.loyalty.dropdown_option"
+54. Select Deduct Points,click,,"admin.customer.loyalty.select_deduct_points"
+55. Enter Points,type,10,"admin.customer.loyalty.input_points"
+56. Click Submit,click,,"web.global.action.submit"
+57. Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+58. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+59. Click Customer Icon,click,,"admin.menu.customer_icon"
+60. Click Verified Customers,click,,"admin.menu.verified_customers"
+61. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+62. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+63. Scroll Grid,tab,7,"admin.customer.filter_name"
+64. Click Disable Icon,click,,"admin.customer.grid.btn_block"
+65. Click Disable User Yes,click,,"web.global.dialog.btn_confirm_yes"
+66. Disable Reason,type,Client Complaints,"web.global.dialog.textarea_reason"
+67. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
+68. Verify Added Successfully,verify,,"web.global.toast.info"
+69. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+70. Click Customer Icon,click,,"admin.menu.customer_icon"
+71. Click Blocked Customers,click,,"admin.menu.blocked_customers"
+72. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+73. Scroll Grid,tab,10,"admin.customer.filter_name"
+74.Wait For Enable Icon,wait_until_visible,,"admin.customer.grid.btn_status_enable"
+75. Click Enable Icon,click,,"admin.customer.grid.btn_status_enable"
+76. Click Enable Yes,click,,"web.global.dialog.btn_confirm_yes"
+77. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+78. Click Customer Icon,click,,"admin.menu.customer_icon"
+79. Click Verified Customers,click,,"admin.menu.verified_customers"
+80. Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+81. Filter Customer Name List,type,{customerName},"admin.customer.filter_name"</t>
   </si>
 </sst>
 </file>
@@ -3520,7 +3522,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>38</v>
@@ -4167,7 +4169,7 @@
         <v>54</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>43</v>
@@ -4243,7 +4245,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>43</v>
@@ -4265,7 +4267,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9466ABF-463D-46B5-A321-4AC4765F1CE7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB63C6AC-3593-403C-90C0-44D30EC92C43}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -4318,7 +4320,7 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
71th Commit: Strore Locator File Created
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1430B7B-3368-4E28-944A-634D6BB3EFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD14C14E-4EE3-469A-A511-DAF31C968419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -22,9 +22,9 @@
     <sheet name="AddTaxiDriver" sheetId="35" r:id="rId7"/>
     <sheet name="TransportServiceCompleteTest" sheetId="37" r:id="rId8"/>
     <sheet name="AddTransportCityAdmin" sheetId="39" r:id="rId9"/>
-    <sheet name="AddStore" sheetId="7" r:id="rId10"/>
-    <sheet name="StoreOperations" sheetId="8" r:id="rId11"/>
-    <sheet name="StoreStatusManagement" sheetId="10" r:id="rId12"/>
+    <sheet name="AddStore" sheetId="40" r:id="rId10"/>
+    <sheet name="StoreOperations" sheetId="42" r:id="rId11"/>
+    <sheet name="StoreStatusManagement" sheetId="43" r:id="rId12"/>
     <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId13"/>
     <sheet name="AddProvider" sheetId="11" r:id="rId14"/>
     <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId15"/>
@@ -331,76 +331,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> The City Area created in the previous AddCityArea must be in an "Active" status to be visible in the cityId dropdown selection.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-RunSheet: AddStore
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
     </r>
   </si>
   <si>
@@ -1449,73 +1379,6 @@
       <t xml:space="preserve">
 </t>
     </r>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-9.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-10.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-11.Click Product Icon,click,,"//i[@title='Product View']"
-12.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
-13.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
-14.Select Grill Chicken,click,,"//li[@role='option'][contains(.,'Grill Chicken')]"
-15.Enter Product Name, type, kfcProduct{randomAlpha}&gt;&gt; kfcProductName, "//label[contains(.,'Product Name')]/following-sibling::input"
-16.Enter Product Amount, type, 500, "//label[contains(.,'Product Amount')]/following-sibling::input"
-17.Enter Product Description, type, KFC special grill chicken, "//label[contains(text(),'Product Description')]/following-sibling::textarea"
-18.Upload Product Image, uploadfile, "src/main/resources/test-data/grillchicken.jpg", "//input[@type='file' and @accept='image/*']"
-19.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[2]"
-20.Select Activate,click,,"//li[@role='option'][contains(.,'Activate')]"
-21.Open Discount Type Dropdown,click,,"//label[contains(.,'Discount Type')]/following-sibling::select/option[text()='Discount in Amount']"
-22.Enter Discount Amount, type, 50, "//label[contains(.,'Discount Amount')]/following-sibling::input"
-23.Click Save, click, , "//button[normalize-space()='Save']"
-24.Verify Saved Succesfully, verify, , "//div[@aria-label='Product added successfully']"
-25.Verify Store Products,verify,,"//div[normalize-space()='Store Products']"
-26.Filter Product List,type,{kfcProductName},"//input[@aria-label='Product Name Filter Input']"
-27.Click Back, click, , "//button[normalize-space()='Back']"
-28.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-29.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-30.Click Wallet Icon,click,,"//i[@title='Wallet']"
-31.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-32.Enter Wallet Amount, type, 1000, "//input[@placeholder='Enter Wallet Amount']"
-33.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-34.Select Add Money,click,,"//li[@role='option' and @aria-label='Add Money']"
-35.Click Submit, click, , "//button[normalize-space()='Submit']"
-36.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-37.Click Manage Transaction, click, , "//button[normalize-space()='Manage Transaction']"
-38.Enter Wallet Amount, type, 200, "//input[@placeholder='Enter Wallet Amount']"
-39.Open Choose Option Dropdown,click,,"//label[contains(.,'Choose Option')]/following-sibling::p-dropdown/div"
-40.Select Deduct Money,click,,"//li[@role='option'][contains(.,'Deduct Money')]"
-41.Click Submit, click, , "//button[normalize-space()='Submit']"
-42.Verify Saved Succesfully, verify, , "//div[@aria-label='Added Successfully']"
-43.Click Back, click, , "//button[normalize-space()='Back']"
-44.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-45.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-46.Click Drivers Icon,click,,"//i[@title='Drivers']"
-47.Click Add Private Driver, click, , "//button[normalize-space()='Add Private Driver']"
-48.Enter Driver Name, type, kfcdriver_{timestamp} &gt;&gt; kfcdriverName, "//label[contains(., 'Driver Full Name')]/following-sibling::div//input"
-49.Enter Email, type, kfcdriver_{timestamp}@gmail.com, "//label[contains(., 'Email')]/following-sibling::div//input"
-50.Enter Contact Number, type, {randomPhone}, "//label[contains(., 'Contact No')]/following-sibling::div//input"
-51.Upload Profile Image, uploadfile, "src/main/resources/test-data/bikedriver.jpg", "//input[@type='file' and @accept='image/*']"
-52. Select Male Gender, click, , "//div[contains(text(), 'Male')]/preceding-sibling::mat-radio-button"
-53.Click Vehicle Type Dropdown,click,,"//label[contains(., 'Vehicle Type')]/following-sibling::p-dropdown"
-54.Select  Scooter Option,click,,"//li[@role='option'][contains(.,'Scooter')]"
-55. Enter Model Year, type, 2013, "//label[span[text()='Model Year']]/following::input[1]"
-56.Enter Vehicle Company, type, kfcBikeCompany{randomAlpha}&gt;&gt; kfcBikeCompanyName, "//label[contains(., 'Vehicle Company')]/following-sibling::div//input"
-57. Enter Plate No, type, KL-01-AB-1634, "//label[contains(., 'Plate No')]/following-sibling::div//input"
-58. Enter Model Name, type, activa, "//label[contains(., 'Model Name')]/following-sibling::div//input"
-59. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/bike.jpg", "(//app-image-upload//input[@type='file'])[2]"
-60. Enter Vehicle Color, type, white, "//label[contains(., 'Vehicle Color')]/following::input[1]"
-61. Click Submit, click, , "//button[contains(.,'Submit')]"
-62. Verify Driver Added, verify, , "//div[@aria-label='Added Successfully']"
-63.Filter Driver List,type,{kfcdriverName},"//input[@aria-label='Driver Name Filter Input']"
-64.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-65.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-secret')]"
@@ -1740,180 +1603,6 @@
   </si>
   <si>
     <t>Super Admin Login</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),'DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-9.Enter Store Name, type, KFC_{timestamp} &gt;&gt; storeName, "//input[@placeholder='Store Name']"
-10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-24.wait,1000,,
-25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-27.wait,1000,,
-28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-34.Enter Contact Person Full Name, type, storeowner_{timestamp} &gt;&gt; storeOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-35.Enter Email, type, kfc_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-41.Enter Accont Holder Name, type, {storeOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-45.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
-46.Enter To Time, type, 100000PM, "((//input[@placeholder='--:--:-- --'])[2])"
-47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-48. Verify Success Message,verify,,"//div[@aria-label='Info']"
-49.Click  Stores,click,,"//button[contains(., 'Stores')]"
-50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-52.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-53.Click  Stores,click,,"//button[contains(., 'Stores')]"
-54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-56.Filter Pending Document Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-63.Click Submit, click, , "//button[normalize-space()='Submit']"
-64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-67.Click Back, click, , "//button[@class='buttonWidget']"
-68.Click  Stores,click,,"//button[contains(., 'Stores')]"
-69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-71.Filter Store List,type,{storeName},"//input[@aria-label='Store Name Filter Input']"
-72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-73.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-74.Click Eye Icon,click,,"//i[@class='bi bi-eye cursor-pointer gridIcon View']"
-75.wait,1000,,</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[contains(@class, 'fa-user-shield')]"
-2.Click Delivery Services,click,,"//h2[contains(text(), 'Delivery Services')]"
-3.Verify Delivery Services,verify,,"//div[contains(text(),' DELIVERY SERVICES')]"
-4.Click Home Icon Food Delivery,click,,"//div[@role='row'][.//span[text()='Food Delivery']]//i[@title='Home']"
-5.Verify Food Delivery Summary,verify,,"//div[normalize-space()='Food Delivery Summary']"
-6.Click  Stores,click,,"//button[contains(., 'Stores')]"
-7.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-8.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-9.Enter Store Name, type, bilal_{timestamp} &gt;&gt; hotelName, "//input[@placeholder='Store Name']"
-10.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-11.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-12.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-13. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-14.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-15.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-16.Enter Short Description, type, KFC is a global fast-food giant famous for its Original Recipe fried chicken, "//input[@placeholder="Type here"]"
-17.Upload Banner Image, uploadfile, "src/main/resources/test-data/kfcbanner.jpg", "//input[@type='file']"
-18.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-19.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-20.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-21.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-22.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-23..Enter Store Address, type, KFC chennai, "//input[@placeholder='Search location']"
-24.wait,1000,,
-25.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-26.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-27.wait,1000,,
-28.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-29.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-30.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-31.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-32.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-33.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-34.Enter Contact Person Full Name, type, bilalowner_{timestamp} &gt;&gt; hotelOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-35.Enter Email, type, bilal_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-36.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-37.Upload Store Image, uploadfile, "src/main/resources/test-data/kfcstore.jpg", "(//input[@type='file'])[2]"
-38.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-39.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-40.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-41.Enter Accont Holder Name, type, {hotelOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-42.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-43.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-44.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-45.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
-46.Enter To Time, type, 100000PM, "((//input[@placeholder='--:--:-- --'])[2])"
-47.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-48. Verify Success Message,verify,,"//div[@aria-label='Info']"
-49.Click  Stores,click,,"//button[contains(., 'Stores')]"
-50.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-51.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-52.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-53.Click  Stores,click,,"//button[contains(., 'Stores')]"
-54.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-55.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-56.Filter Pending Document Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-57.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-58.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-59. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-60.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-61.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-62.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-63.Click Submit, click, , "//button[normalize-space()='Submit']"
-64.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-65.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-66.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-67.Click Back, click, , "//button[@class='buttonWidget']"
-68.Click  Stores,click,,"//button[contains(., 'Stores')]"
-69.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-70.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-71.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-72.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-73.Click Block Icon,click,,"//i[@title='Blocked']"
-74.Click Block  Yes,click,,"//button[normalize-space()='Yes']"
-75.Click  Stores,click,,"//button[contains(., 'Stores')]"
-76.Select Blocked Store,click,,"//div[normalize-space()='Blocked Stores']"
-77.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-78.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-79.Click unBlock Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-80.Click  Stores,click,,"//button[contains(., 'Stores')]"
-81.Select Rejected Store,click,,"//div[normalize-space()='Rejected Stores']"
-82.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-83.Scroll Grid, tab, 7, "//input[@aria-label='Store Name Filter Input']"
-84.Click Approve Icon,click,,"//i[@title='Approve']"
-85.Click  Stores,click,,"//button[contains(., 'Stores')]"
-86.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-87.Filter Store List,type,{hotelName},"//input[@aria-label='Store Name Filter Input']"
-88.wait,3000,,
-89.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-90.Click Doc Icon,click,,"//i[@title='Document']"
-91.Click UnApprove Icon,click,,"//i[@class='bi bi-hand-thumbs-down-fill cursor-pointer gridIcon Modify']"
-92.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-93.Rejection Reason,type,document insufficent,"//textarea[@id='swal2-textarea']"
-94.Click Reject  Yes,click,,"//button[normalize-space()='Yes']"
-95.wait,1000,,</t>
   </si>
   <si>
     <t>1.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
@@ -3130,6 +2819,321 @@
 35.Click Submit,click,,"web.global.login.submit_btn"
 36. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
 37.Filter admin name,type,{adminName},"admin.city_admin.input_name_filter"</t>
+  </si>
+  <si>
+    <t>1. Click badge,click,,"admin.store.badge.shield"
+2. Click Delivery Services,click,,"admin.store.delivery_services.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.store.delivery_services.header"
+4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
+5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
+6. Click Stores,click,,"admin.store.menu.toggle_btn"
+7. Select Add Store,click,,"admin.store.submenu.add_store"
+8. Wait For Add Store,wait_until_visible,,"admin.store.add_page.header"
+9. Enter Store Name,type,KFC_{timestamp} &gt;&gt; storeName,"admin.store.name.input"
+10. Open Delivery Radius Dropdown,click,,"admin.store.radius.dropdown"
+11. Select Twenty Five Kilometer,click,,"admin.store.radius.option_25km"
+12. Open Estimated Delivery Time,click,,"admin.store.eta.dropdown"
+13. Select Thirty Minute,click,,"admin.store.eta.option_30min"
+14. Enter Order Minimum Amount,type,300,"admin.store.min_amount.input"
+15. Enter Packaging Charges,type,50,"admin.store.packaging_charge.input"
+16. Enter Short Description,type,KFC is a global fast-food giant famous for its Original Recipe fried chicken,"admin.store.description.input"
+17. Upload Banner Image,uploadfile,"src/main/resources/test-data/kfcbanner.jpg","admin.store.banner.file"
+18. Open Driver Notification,click,,"admin.store.driver_notification.dropdown"
+19. Select Both Driver,click,,"admin.store.driver_notification.option_both"
+20. Click Checkbox Allow For Pickup,click,,"admin.store.allow_pickup.checkbox"
+21. Open Current Status Dropdown,click,,"admin.store.current_status.dropdown"
+22. Select Active,click,,"admin.store.current_status.option_active"
+23. Enter Store Address,type,KFC chennai,"admin.store.location.input"
+24. wait,3000,,
+25. Confirm Store Address,press_enter,,"admin.store.location.input"
+26. wait,3000,,
+27. Select First Option,arrow_down,,"admin.store.location.input"
+28. Confirm Option,press_enter,,"admin.store.location.input"
+29. wait,2000,,
+30. Click Storewise Comission Checkbox,click,,"admin.store.commission.checkbox"
+31. Enter Store Commision,type,25,"admin.store.commission_rate.input"
+32. Open Driver Notification,click,,"admin.store.offer_type.dropdown"
+33. Select Amount,click,,"admin.store.offer_type.option_amount"
+34. Enter Offer Amount,type,50,"admin.store.offer_amount.input"
+35. Enter Offer Min Amount,type,500,"admin.store.offer_min_amount.input"
+36. Enter Contact Person Full Name,type,storeowner_{timestamp} &gt;&gt; storeOwner,"admin.store.contact_name.input"
+37. Enter Email,type,kfc_{timestamp}@gmail.com&gt;&gt;storeEmail,"admin.store.email.input"
+38. Enter Contact Number,type,{randomPhone},"admin.store.phone.input"
+39. Upload Store Image,uploadfile,"src/main/resources/test-data/kfcstore.jpg","admin.store.profile.file"
+40. Enter Bank Name,type,federal,"admin.store.bank.name_input"
+41. Enter Bank Location,type,chennai,"admin.store.bank.location_input"
+42. Enter Account Number,type,123456789012,"admin.store.bank.account_input"
+43. Enter Accont Holder Name,type,{storeOwner},"admin.store.bank.holder_input"
+44. Enter Payment Email Address,type,{storeEmail},"admin.store.bank.payment_email"
+45. Enter BIC Code,type,1234,"admin.store.bank.bic_input"
+46. Click Store Timing Checkbox,click,,"admin.store.timing.everyday_checkbox"
+47. Enter From Time,type,100000AM,"admin.store.timing.from_input"
+48. Enter To Time,type,100000PM,"admin.store.timing.to_input"
+49. Submit Add Store,click,,"web.global.action.submit"
+50. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
+51. Click Stores,click,,"admin.store.menu.toggle_btn"
+52. Select Store List,click,,"admin.store.submenu.store_list"
+53. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+54. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+55. Click Stores,click,,"admin.store.menu.toggle_btn"
+56. Select Pending Documents Stores List,click,,"admin.store.submenu.pending_docs"
+57. Wait For Add Store,wait_until_visible,,"admin.store.pending_page.header"
+58. Filter Pending Document Store List,type,{storeName},"admin.store.grid.name_filter"
+59. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+60. Click Doc Icon,click,,"admin.store.grid.doc_icon"
+61. Store Required Documents,verify,,"admin.store.documents_page.header"
+62. Add Address Proof,click,,"admin.store.grid.edit_doc_icon"
+63. Upload Address Proof,uploadfile,"src/main/resources/test-data/addressproof.png","admin.store.doc.file_input"
+64. Enter Expiry Date,type,2026-12-12,"admin.store.doc.expiry_input"
+65. Click Submit,click,,"web.global.action.submit"
+66. Verify Updated Succesfully,verify,,"web.global.toast.updated"
+67. Click Approve Store,click,,"admin.store.grid.approve_doc_icon"
+68. Verify Updated Succesfully,verify,,"web.global.toast.updated"
+69. Click Back,click,,"admin.store.grid.back_btn"
+70. Click Stores,click,,"admin.store.menu.toggle_btn"
+71. Select Store List,click,,"admin.store.submenu.store_list"
+72. Verify Add Store,verify,,"admin.store.list_page.header"
+73. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+74. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+75. Click Doc Icon,click,,"admin.store.grid.doc_icon"
+76. Click Eye Icon,click,,"admin.store.grid.eye_view_icon"
+77. wait,1000,,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+RunSheet: AddStore2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Click badge,click,,"admin.store.badge.shield"
+2. Click Delivery Services,click,,"admin.store.delivery_services.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.store.delivery_services.header"
+4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
+5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
+6. Click Stores,click,,"admin.store.menu.toggle_btn"
+7. Select Store List,click,,"admin.store.submenu.store_list"
+8. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+9. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+10. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+11. Click Product Icon,click,,"admin.store.products.grid_icon"
+12. Click Add Products,click,,"admin.store.products.add_btn"
+13. Open Product Category Dropdown,click,,"admin.store.products.category_dropdown"
+14. Select Grill Chicken,click,,"admin.store.products.category_option_grill"
+15. Enter Product Name,type,kfcProduct{randomAlpha}&gt;&gt; kfcProductName,"admin.store.products.name_input"
+16. Enter Product Amount,type,500,"admin.store.products.amount_input"
+17. Enter Product Description,type,KFC special grill chicken,"admin.store.products.description_textarea"
+18. Upload Product Image,uploadfile,"src/main/resources/test-data/grillchicken.jpg","admin.store.products.image.file"
+19. Open Product Category Dropdown,click,,"admin.store.products.status_dropdown"
+20. Select Activate,click,,"admin.store.products.status_option_active"
+21. Open Discount Type Dropdown,click,,"admin.store.products.discount_dropdown"
+22. Enter Discount Amount,type,50,"admin.store.products.discount_input"
+23. Click Save,click,,"admin.store.products.save_btn"
+24. Wait For Saved Succesfully,wait_until_visible,,"admin.store.products.toast_success"
+25. Wait For Store Products,wait_until_visible,,"admin.store.products.header"
+26. Filter Product List,type,{kfcProductName},"admin.store.products.name_filter"
+27. Click Back,click,,"admin.store.products.back_btn"
+28. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+29. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+30. Click Wallet Icon,click,,"admin.store.wallet.grid_icon"
+31. Click Manage Transaction,click,,"admin.store.wallet.manage_transaction_btn"
+32. Enter Wallet Amount,type,1000,"admin.store.wallet.amount_input"
+33. Open Choose Option Dropdown,click,,"admin.store.wallet.option_dropdown"
+34. Select Add Money,click,,"admin.store.wallet.option_add"
+35. Click Submit,click,,"web.global.action.submit"
+36. Wait For Saved Succesfully,wait_until_visible,,"web.global.toast.success"
+37. Click Manage Transaction,click,,"admin.store.wallet.manage_transaction_btn"
+38. Enter Wallet Amount,type,200,"admin.store.wallet.amount_input"
+39. Open Choose Option Dropdown,click,,"admin.store.wallet.option_dropdown"
+40. Select Deduct Money,click,,"admin.store.wallet.option_deduct"
+41. Click Submit,click,,"web.global.action.submit"
+42. Wait For Saved Succesfully,wait_until_visible,,"web.global.toast.success"
+43. Click Back,click,,"admin.store.products.back_btn"
+44. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+45. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+46. Click Drivers Icon,click,,"admin.store.drivers.grid_icon"
+47. Click Add Private Driver,click,,"admin.store.drivers.add_private_btn"
+48. Enter Driver Name,type,kfcdriver_{timestamp} &gt;&gt; kfcdriverName,"admin.drivers.fullname.input"
+49. Enter Email,type,kfcdriver_{timestamp}@gmail.com,"admin.drivers.email.input"
+50. Enter Contact Number,type,{randomPhone},"admin.drivers.phone.input"
+51. Upload Profile Image,uploadfile,"src/main/resources/test-data/bikedriver.jpg","admin.drivers.profile_image.file"
+52. Select Male Gender,click,,"admin.drivers.male_gender.div"
+53. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+54. Select Scooter Option,click,,"admin.drivers.vehicle_option.scooter"
+55. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
+56. Enter Vehicle Company,type,kfcBikeCompany{randomAlpha}&gt;&gt; kfcBikeCompanyName,"admin.drivers.companyname.input"
+57. Enter Plate No,type,KL-01-AB-1634,"admin.drivers.plateno.input"
+58. Enter Model Name,type,activa,"admin.drivers.modelname.input"
+59. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/bike.jpg","admin.drivers.vehicle_image.file"
+60. Enter Vehicle Color,type,white,"admin.drivers.vehicle_color.input"
+61. Click Submit,click,,"web.global.action.submit"
+62. Wait For Driver Added,wait_until_visible,,"web.global.toast.success"
+63. Filter Driver List,type,{kfcdriverName},"admin.drivers.name_filter.input"
+64. Click Eye Icon,click,,"admin.store.grid.eye_view_icon"
+65. wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click badge,click,,"admin.store.badge.shield"
+2. Click Delivery Services,click,,"admin.store.delivery_services.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.store.delivery_services.header"
+4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
+5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
+6. Click Stores,click,,"admin.store.menu.toggle_btn"
+7. Select Add Store,click,,"admin.store.submenu.add_store"
+8. Wait For Add Store,wait_until_visible,,"admin.store.add_page.header"
+9. Enter Store Name,type,bilal_{timestamp} &gt;&gt; hotelName,"admin.store.name.input"
+10. Open Delivery Radius Dropdown,click,,"admin.store.radius.dropdown"
+11. Select Twenty Five Kilometer,click,,"admin.store.radius.option_25km"
+12. Open Estimated Delivery Time,click,,"admin.store.eta.dropdown"
+13. Select Thirty Minute,click,,"admin.store.eta.option_30min"
+14. Enter Order Minimum Amount,type,300,"admin.store.min_amount.input"
+15. Enter Packaging Charges,type,50,"admin.store.packaging_charge.input"
+16. Enter Short Description,type,KFC is a global fast-food giant famous for its Original Recipe fried chicken,"admin.store.description.input"
+17. Upload Banner Image,uploadfile,"src/main/resources/test-data/kfcbanner.jpg","admin.store.banner.file"
+18. Open Driver Notification,click,,"admin.store.driver_notification.dropdown"
+19. Select Both Driver,click,,"admin.store.driver_notification.option_both"
+20. Click Checkbox Allow For Pickup,click,,"admin.store.allow_pickup.checkbox"
+21. Open Current Status Dropdown,click,,"admin.store.current_status.dropdown"
+22. Select Active,click,,"admin.store.current_status.option_active"
+23. Enter Store Address,type,KFC chennai,"admin.store.location.input"
+24. wait,3000,,
+25. Confirm Store Address,press_enter,,"admin.store.location.input"
+26. wait,3000,,
+27. Select First Option,arrow_down,,"admin.store.location.input"
+28. Confirm Option,press_enter,,"admin.store.location.input"
+29. wait,2000,,
+30. Click Storewise Comission Checkbox,click,,"admin.store.commission.checkbox"
+31. Enter Store Commision,type,25,"admin.store.commission_rate.input"
+32. Open Driver Notification,click,,"admin.store.offer_type.dropdown"
+33. Select Amount,click,,"admin.store.offer_type.option_amount"
+34. Enter Offer Amount,type,50,"admin.store.offer_amount.input"
+35. Enter Offer Min Amount,type,500,"admin.store.offer_min_amount.input"
+36. Enter Contact Person Full Name,type,bilalowner_{timestamp} &gt;&gt; hotelOwner,"admin.store.contact_name.input"
+37. Enter Email,type,bilal_{timestamp}@gmail.com&gt;&gt;storeEmail,"admin.store.email.input"
+38. Enter Contact Number,type,{randomPhone},"admin.store.phone.input"
+39. Upload Store Image,uploadfile,"src/main/resources/test-data/kfcstore.jpg","admin.store.profile.file"
+40. Enter Bank Name,type,federal,"admin.store.bank.name_input"
+41. Enter Bank Location,type,chennai,"admin.store.bank.location_input"
+42. Enter Account Number,type,123456789012,"admin.store.bank.account_input"
+43. Enter Accont Holder Name,type,{hotelOwner},"admin.store.bank.holder_input"
+44. Enter Payment Email Address,type,{storeEmail},"admin.store.bank.payment_email"
+45. Enter BIC Code,type,1234,"admin.store.bank.bic_input"
+46. Click Store Timing Checkbox,click,,"admin.store.timing.everyday_checkbox"
+47. Enter From Time,type,100000AM,"admin.store.timing.from_input"
+48. Enter To Time,type,100000PM,"admin.store.timing.to_input"
+49. Submit Add Store,click,,"web.global.action.submit"
+50. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
+51. Click Stores,click,,"admin.store.menu.toggle_btn"
+52. Select Store List,click,,"admin.store.submenu.store_list"
+53. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+54. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+55. Click Stores,click,,"admin.store.menu.toggle_btn"
+56. Select Pending Documents Stores List,click,,"admin.store.submenu.pending_docs"
+57. Wait For Add Store,wait_until_visible,,"admin.store.pending_page.header"
+58. Filter Pending Document Store List,type,{hotelName},"admin.store.grid.name_filter"
+59. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+60. Click Doc Icon,click,,"admin.store.grid.doc_icon"
+61. Wait For Store Required Documents,wait_until_visible,,"admin.store.documents_page.header"
+62. Add Address Proof,click,,"admin.store.grid.edit_doc_icon"
+63. Upload Address Proof,uploadfile,"src/main/resources/test-data/addressproof.png","admin.store.doc.file_input"
+64. Enter Expiry Date,type,2026-12-12,"admin.store.doc.expiry_input"
+65. Click Submit,click,,"web.global.action.submit"
+66. Wait For Updated Succesfully,wait_until_visible,,"web.global.toast.updated"
+67. Click Approve Store,click,,"admin.store.grid.approve_doc_icon"
+68. Verify Updated Succesfully,verify,,"web.global.toast.updated"
+69. Click Back,click,,"admin.store.grid.back_btn"
+70. Click Stores,click,,"admin.store.menu.toggle_btn"
+71. Select Store List,click,,"admin.store.submenu.store_list"
+72. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+73. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+74. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+75. Click Block Icon,click,,"admin.store.grid.block_icon"
+76. Click Block Yes,click,,"web.global.dialog.btn_confirm_yes"
+77. Click Stores,click,,"admin.store.menu.toggle_btn"
+78. Select Blocked Store,click,,"admin.store.submenu.blocked_stores"
+79. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+80. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+81. Click unBlock Icon,click,,"admin.store.grid.unblock_icon"
+82. Click Stores,click,,"admin.store.menu.toggle_btn"
+83. Select Rejected Store,click,,"admin.store.submenu.rejected_stores"
+84. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+85. Scroll Grid,tab,7,"admin.store.grid.name_filter"
+86. Click Approve Icon,click,,"admin.store.grid.approve_icon"
+87. Click Stores,click,,"admin.store.menu.toggle_btn"
+88. Select Store List,click,,"admin.store.submenu.store_list"
+89. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+90. wait,3000,,
+91. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+92. Click Doc Icon,click,,"admin.store.grid.document_icon"
+93. Click UnApprove Icon,click,,"admin.store.grid.unapprove_icon"
+94. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
+95. Rejection Reason,type,document insufficent,"web.global.dialog.textarea_reason"
+96. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
+97. wait,1000,,</t>
   </si>
 </sst>
 </file>
@@ -3546,7 +3550,7 @@
         <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -3555,7 +3559,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -3577,7 +3581,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C456A73-57BC-411E-B40E-DADED30882CB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9950CA5-B845-4E23-9843-8D459D399E99}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3624,16 +3628,16 @@
         <v>27</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3649,7 +3653,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86A4538F-421E-4B0B-A965-0382A5BEF523}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DE0E168-E98A-49FE-8885-7B5F3F3678F3}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3690,22 +3694,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>69</v>
+        <v>114</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>39</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3721,7 +3725,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57207608-1AD9-408F-B018-55A141C9A651}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9584B63-AFDB-41EC-A160-356B47922D15}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3762,22 +3766,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>77</v>
+        <v>115</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3834,22 +3838,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3906,22 +3910,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3978,22 +3982,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4050,22 +4054,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4122,22 +4126,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4189,7 +4193,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4200,22 +4204,22 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="D2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4282,16 +4286,16 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4343,7 +4347,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4357,19 +4361,19 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -4411,7 +4415,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4425,19 +4429,19 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4486,7 +4490,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4500,19 +4504,19 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4561,7 +4565,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4575,19 +4579,19 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4636,7 +4640,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4647,22 +4651,22 @@
         <v>29</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4720,22 +4724,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
71th Commit: Delievery Service Locator File Created
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD14C14E-4EE3-469A-A511-DAF31C968419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BF513C-6185-45BE-8062-0F8880287EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <sheet name="AddStore" sheetId="40" r:id="rId10"/>
     <sheet name="StoreOperations" sheetId="42" r:id="rId11"/>
     <sheet name="StoreStatusManagement" sheetId="43" r:id="rId12"/>
-    <sheet name="DeliveryServiceCompleteTest" sheetId="14" r:id="rId13"/>
+    <sheet name="DeliveryServiceCompleteTest" sheetId="44" r:id="rId13"/>
     <sheet name="AddProvider" sheetId="11" r:id="rId14"/>
     <sheet name="ProviderServiceCompleteTest" sheetId="12" r:id="rId15"/>
     <sheet name="SubscriptionPlanTest" sheetId="29" r:id="rId16"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="120">
   <si>
     <t>City Area</t>
   </si>
@@ -1603,177 +1603,6 @@
   </si>
   <si>
     <t>Super Admin Login</t>
-  </si>
-  <si>
-    <t>1.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
-2.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
-3.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
-4.Click  Add Service Category,click,,"//button[normalize-space()='Add Service Category']"
-5.Enter Category Name, type, milk Delivery{randomAlpha}&gt;&gt; deliveryName, "//input[@placeholder='Category Name']"
-6.Enter Slug, type, Milk Delivery, "//input[@placeholder='Slug']"
-7.Upload Category Image, uploadfile, "src/main/resources/test-data/milkman.jpg", "//input[@type='file' and @accept='image/*']"
-8.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-9.Select Activate,click,,"//li[@aria-label='Activate']"
-10.Open Category Flow Dropdown,click,,"//label[contains(., 'Category Flow')]/following-sibling::p-dropdown"
-11.Select default flow(food-delivery),click,,"//li[@aria-label='default flow(food-delivery)']"
-12.Enter Delivery Name Tamil, type,பால்காரர், "//input[@placeholder='Enter in Tamil']"
-13.Enter Delivery Name Arabic, type, لبّان, "//input[@placeholder='Enter in Arabic']"
-14.Enter Delivery Name Hindi, type, दूधवाला, "//input[@placeholder='Enter in Hindi']"
-15.Click  Submit,click,,"//button[normalize-space()='Submit']"
-16.Verify Sucess, verify, , "//div[@aria-label='Info']"
-17.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
-18.Click Home Icon ,click,,"//i[@title='Home']"
-19.Click Settings ,click,,"//button[contains(., 'Settings')]"
-20.Click Requirment Document ,click,,"//div[contains(text(), 'Required Documents')]"
-21.Click Add Document ,click,,"//button[normalize-space()='Add Document']"
-22.Enter Name, type, documet{randomAlpha}&gt;&gt; deliveryDocumentName, "//input[@placeholder='Type here']"
-23.Open status Dropdown,click,,"//span[@aria-label='select status']"
-24.Select Active,click,,"//li[@aria-label='Active']"
-25.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-26.Click Document Expiry ,click,,"//div[./div[contains(text(), 'Document Expiry')]]//input"
-27.Click Mandatory Document ,click,,"//div[./div[contains(text(), 'Mandatory Document')]]//input"
-28.Click  Require Proof Number,click,,"//div[./div[contains(text(), 'Require Proof Number')]]//input"
-29.Enter Display Order, type, 10,"//input[@placeholder='Display Order']"
-30.Click Submit ,click,,"//button[normalize-space()='Submit']"
-31.Verify Sucess, verify, , "//div[@aria-label='Info']"
-32.Filter Document List,type,{deliveryDocumentName},"//input[@aria-label='Name Filter Input']"
-33.wait,2000,,
-33.Click Settings ,click,,"//button[contains(., 'Settings')]"
-34.Click Promocode ,click,,"//div[normalize-space()='Promocode']"
-35.Click Add Promo Code ,click,,"//button[normalize-space()='Add Promo Code']"
-36.Open User List Dropdown,click,,"//label[contains(., 'User List')]/following-sibling::p-multiselect//div[contains(@class, 'p-multiselect-label-container')]"
-37.Select User,click,,"//li[@aria-label='{customerName}']"
-38.Click Code Name Box,click,,"//input[@placeholder='Code Name']"
-39.Enter Code Name, type, promoCode{randomAlpha}&gt;&gt; deliveryPromoCodeName, "//input[@placeholder='Code Name']"
-40.Open Discout Type Dropdown,click,,"//span[@aria-label='Select Discount Type']"
-41.Select Discout Type,click,,"//li[@aria-label='Discount in Amount ']"
-42.Enter Expiry Date,type,12122026,"//div[label[contains(., 'Expiry Date')]]//input"
-43.Enter Discount Amount, type, 100, "//input[@placeholder='Discount Amount']"
-44.Enter Minimum Order Amount, type, 1000, "//input[@placeholder='Min Order Amount']"
-45.Enter Maximum Discount Amount, type, 100, "//input[@placeholder='Max DiscountAmount']"
-46.Enter Coupon Limit, type, 5,"//div[label[contains(., 'Coupon Limit')]]//input"
-47.Enter Usage Limit for One User, type, 2,"//div[label[contains(., 'Usage Limit For One User')]]//input"
-48.Enter Promo Code Description, type, Promo Dode For Gold Member,"//textarea[@placeholder='PromoCode Description']"
-49.Click Submit ,click,,"//button[normalize-space()='Submit']"
-50.Verify Sucess, verify, , "//div[@aria-label='Info']"
-51.Filter PromoCode List,type,{deliveryPromoCodeName},"//input[@aria-label='promocode Filter Input']"
-52.wait,2000,,
-53.Click Settings ,click,,"//button[contains(., 'Settings')]"
-54.Click Service Settings ,click,,"//div[normalize-space()='Service Settings']"
-55.Enter Driver Serach Radius, type, 50, "//span[contains(text(), 'Driver search Radius')]/ancestor::app-input//input"
-56.Open Tax Type Dropdown,click,,"//span[@aria-label='Select Tax Type']"
-57.Select Amount,click,,"//li[@aria-label='Amount']"
-58.Enter Tax, type, 20, "//span[contains(text(), 'Tax')]/ancestor::app-input//input"
-59.Open Platform Fee Type Dropdown,click,,"//span[@aria-label='Seelct Type']"
-60.Select Amount,click,,"//li[@aria-label='Amount']"
-61.Enter Platform Fee, type, 20, "//span[contains(text(), 'Platform Fee')]/ancestor::app-input//input"
-62.Enter Cancel Charge (in %):, type, 20, "//span[contains(text(), 'Cancel Charge (in %):')]/ancestor::app-input//input"
-63.Enter Driver Accept Timeout (in Second):, type, 20, "//span[contains(text(), 'Driver Accept Timeout (in Second):')]/ancestor::app-input//input"
-64.Click Submit ,click,,"//button[normalize-space()='Submit']"
-65.Verify Sucess, verify, , "//div[@aria-label='Info']"
-66.Click  Stores,click,,"//button[contains(., 'Stores')]"
-67.Select Add Store,click,,"//div[contains(text(), 'Add Store')]"
-68.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Add Store')]"
-69.Enter Store Name, type, amul_{timestamp} &gt;&gt; milkStore, "//input[@placeholder='Store Name']"
-70.Open Delivery Radius Dropdown,click,,"//span[@aria-label='select radius']"
-71.Select Twenty Five Kilometer,click,,"//li[@role='option'][contains(.,'25 KM')]"
-72.Open Estimated Delivery Time,click,,"//span[@aria-label='Estimated Delivery Time']"
-73. Select Thirty Minute,click,,"//li[@role='option'][contains(.,'30 MIN')]"
-74.Enter Order Minimum Amount, type, 300, "//input[@placeholder='Order Min Amount']"
-75.Enter Packaging Charges, type, 50, "//input[@placeholder='Packaging Charges']"
-76.Enter Short Description, type, amul taste of india, "//input[@placeholder="Type here"]"
-77.Upload Banner Image, uploadfile, "src/main/resources/test-data/amulbanner.jpg", "//input[@type='file']"
-78.Open Driver Notification,click,,"//span[@aria-label='select driver type']"
-79.Select Both Driver,click,,"//li[@role='option'][contains(.,'Both Driver')]"
-80.Click Checkbox Allow For Pickup , click, , "//label[contains(., "Do You Want ?")]/following-sibling::div//mat-checkbox"
-81.Open Current Status Dropdown,click,,"//span[@aria-label='Active']"
-82.Select Active,click,,"//li[@role='option'][contains(.,'Active')]"
-83..Enter Store Address, type, Amul chennai, "//input[@placeholder='Search location']"
-84.wait,1000,,
-85.Select First Option,arrow_down,,"//input[@placeholder='Search location']"
-86.Confirm Option,press_enter,,"//input[@placeholder='Search location']"
-87.wait,1000,,
-88.Click Storewise Comission Checkbox, click, , "//div[contains(text(),'Store Wise Commission')]/preceding-sibling::mat-checkbox"
-89.Enter Store Commision, type, 25, "//label[contains(.,'Commission (in %)')]/following-sibling::div//input"
-90.Open Driver Notification,click,,"//span[@aria-label='select offer type']"
-91.Select Amount,click,,"//li[@role='option'][contains(.,'Amount')]"
-92.Enter Offer Amount, type, 50, "//label[contains(.,'Offer Amount')]/following-sibling::div//input"
-93.Enter Offer Min Amount, type, 500, "//label[contains(.,'Offer Min Amount')]/following-sibling::div//input"
-94.Enter Contact Person Full Name, type, amulStoreowner_{timestamp} &gt;&gt; milkStoreOwner, "//label[contains(.,'Contact Person Full Name')]/following-sibling::div//input"
-95.Enter Email, type, amul_{timestamp}@gmail.com&gt;&gt;storeEmail, "//label[contains(.,'Email Address')]/following-sibling::div//input"
-96.Enter Contact Number, type, {randomPhone}, "//label[contains(.,'Contact Number')]/following-sibling::div//input"
-97.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "(//input[@type='file'])[2]"
-98.Enter Bank Name, type, federal, "//label[contains(.,'Bank Name')]/following-sibling::div//input"
-99.Enter Bank Location,type, chennai, "//label[contains(.,'Bank Location(City Name)')]/following-sibling::div//input"
-100.Enter Account Number, type, 123456789012, "//label[contains(.,'Account Number')]/following-sibling::div//input"
-101.Enter Accont Holder Name, type, {milkStoreOwner}, "//label[contains(.,'Account Holder Name')]/following-sibling::div//input"
-102.Enter Payment Email Address, type, {storeEmail}, "//label[contains(.,'Payment Email Address')]/following-sibling::div//input"
-103.Enter BIC Code, type, 1234, "//label[contains(.,'BIC Code')]/following-sibling::div//input"
-104.Click Store Timing Checkbox, click, , "//div[contains(text(),'Every Day')]/preceding-sibling::mat-checkbox"
-105.Enter From Time, type, 100000AM, "((//input[@placeholder='--:--:-- --'])[1])"
-106.Enter To Time, type, 100000PM, "((//input[@placeholder='--:--:-- --'])[2])"
-107.Submit Add Store,click,,"//button[normalize-space()='Submit']"
-108. Verify Success Message,verify,,"//div[@aria-label='Info']"
-109.Click  Stores,click,,"//button[contains(., 'Stores')]"
-110.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-111.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-112.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-113.Click  Stores,click,,"//button[contains(., 'Stores')]"
-114.Select Pending Documents Stores List,click,,"//div[contains(text(), 'Pending Documents Stores')]"
-115.Verify Add Store,verify,,"//div[normalize-space()='Pending Documents Store']"
-116.Filter Pending Document Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-117.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-118.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-119. Store Required Documents,verify,,"//div[contains(text(),'Documents')]"
-120.Add Address Proof,click,,"//i[@class='bi bi-pencil-square cursor-pointer gridIcon Edit']"
-121.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "//input[@type='file']"
-122.Enter Expiry Date,type,2026-12-12,"//input[@placeholder='YYYY/MM/DD']"
-123.Click Submit, click, , "//button[normalize-space()='Submit']"
-124.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-125.Click Approve Store,click,,"//i[@class='bi bi-hand-thumbs-up-fill cursor-pointer gridIcon Modify']"
-126.Verify Updated Succesfully, verify, , "//div[@aria-label='Updated Successfully']"
-127.Click Back, click, , "//button[@class='buttonWidget']"
-128.Click  Stores,click,,"//button[contains(., 'Stores')]"
-129.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-130.Verify Add Store,verify,,"//app-text[@class='ng-star-inserted']//div[contains(text(),'Store List')]"
-131.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-132.Scroll Grid, tab, 8, "//input[@aria-label='Store Name Filter Input']"
-133.Click Doc Icon,click,,"//i[contains(@class, 'bi-file-earmark-medical-fill') and contains(@class, 'Navigate')]"
-134.Click Back, click, , "//button[@class='buttonWidget']"
-135.Click Category, click, , "//button[normalize-space()='Category']"
-136.Click  Add New Category,click,,"//button[normalize-space()='Add Category']"
-137.Enter Category Name, type,curd{randomAlpha}&gt;&gt; MilkCategoryName, "//span[contains(text(), 'Category Name')]/ancestor::app-input//input"
-138.Enter Category Name Arabic, type, رائب, "//span[contains(text(), 'Language Value (in Arabic)')]/ancestor::app-input//input"
-139.Enter Category Name Tamil, type, தயிர், "//span[contains(text(), 'Language Value (in Tamil)')]/ancestor::app-input//input"
-140.Enter Category Name Hindi, type, दही, "//span[contains(text(), 'Language Value (in Hindi)')]/ancestor::app-input//input"
-141.Open Category status Dropdown,click,,"//span[@aria-label='status']"
-142.Select Active,click,,"//li[@aria-label='active']"
-143.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "//input[@type='file' and @accept='image/*']"
-144.wait,2000,,
-145.Enter Slug Name, type, curd, "//span[text()='Slug']/ancestor::app-input//input"
-146.Click  Submit,click,,"//button[normalize-space()='Submit']"
-147.Verify Success Message,verify,,"//div[@aria-label='Info']"
-148.Filter Category Name,type,{MilkCategoryName},"//input[@aria-label='Category Name Filter Input']"
-149.Click  Stores,click,,"//button[contains(., 'Stores')]"
-150.Select Store List,click,,"//div[contains(text(), 'Store List')]"
-151.Filter Store List,type,{milkStore},"//input[@aria-label='Store Name Filter Input']"
-152.Scroll Grid, tab, 9, "//input[@aria-label='Store Name Filter Input']"
-153.Click Product Icon,click,,"//i[@title='Product View']"
-154.Click  Add  Products,click,,"//button[normalize-space()='Add Products']"
-155.Open Product Category Dropdown,click,,"(//label[contains(text(),'Product Category')]/following-sibling::p-dropdown/div)[1]"
-156.Select curd,click,,"//li[@role='option'][contains(.,'{MilkCategoryName}')]"
-157.wait,1000,,
-158.Click badge,click,,"//i[@class='fa-solid fa-user-shield iconstyle']"
-159.Click Delivery Services,click,,"//h2[normalize-space()='Delivery Services']"
-160.Verify Delivery Services,verify,,"//div[normalize-space()='DELIVERY SERVICES']"
-161.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
-162.Click Edit Icon ,click,,"//i[@title='Edit']"
-163.Open status Dropdown,click,,"//label[contains(., 'Status')]/following-sibling::p-dropdown"
-164.wait,1000,,
-164.Select Dectivate,click,,"//li[@aria-label='Deactivate']"
-165.Click Submit ,click,,"//button[normalize-space()='Submit']"
-166.Filter Services List,type,{deliveryName},"//input[@aria-label='Services Filter Input']"
-167.wait,1000,,</t>
   </si>
   <si>
     <t xml:space="preserve">1.Click badge,click,,"//i[contains(@class, 'fa-hand-holding-usd fa-solid iconstyle')]"
@@ -2821,9 +2650,433 @@
 37.Filter admin name,type,{adminName},"admin.city_admin.input_name_filter"</t>
   </si>
   <si>
-    <t>1. Click badge,click,,"admin.store.badge.shield"
-2. Click Delivery Services,click,,"admin.store.delivery_services.menu"
-3. Wait For Delivery Services,wait_until_visible,,"admin.store.delivery_services.header"
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Data Dependency: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
+RunSheet: AddStore2
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Authentication State: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Navigation State:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Actual Test Steps</t>
+  </si>
+  <si>
+    <t>1.Click badge, click, , "admin.store.badge.shield"
+2.Click Delivery Services, click, , "admin.store.delivery_services.menu"
+3.Verify Delivery Services, verify, , "admin.store.delivery_services.header"
+4.Click Add Service Category, click, , "admin.deliveryservice.add_category_btn"
+5.Enter Category Name, type, milk Delivery{randomAlpha} &gt;&gt; deliveryName, "admin.deliveryservice.category_name.input"
+6.Enter Slug, type, Milk Delivery, "admin.deliveryservice.slug.input"
+7.Upload Category Image, uploadfile, "src/main/resources/test-data/milkman.jpg", "admin.deliveryservice.image.file"
+8.Open status Dropdown, click, , "admin.deliveryservice.status.dropdown"
+9.Select Activate, click, , "admin.deliveryservice.status.option_activate"
+10.Open Category Flow Dropdown, click, , "admin.deliveryservice.flow.dropdown"
+11.Select default flow(food-delivery), click, , "admin.deliveryservice.flow.option_food_delivery"
+12.Enter Delivery Name Tamil, type, பால்காரர், "admin.deliveryservice.lang_tamil.input"
+13.Enter Delivery Name Arabic, type, لبّان, "admin.deliveryservice.lang_arabic.input"
+14.Enter Delivery Name Hindi, type, दूधवाला, "admin.deliveryservice.lang_hindi.input"
+15.Click Submit, click, , "web.global.action.submit"
+16.Verify Success, verify, , "web.global.toast.info"
+17.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+18.Click Home Icon, click, , "admin.store.food_delivery.home_icon"
+19.Click Settings, click, , "admin.deliveryservice.menu.toggle_btn"
+20.Click Requirement Document, click, , "admin.deliveryservice.submenu.required_docs"
+21.Click Add Document, click, , "admin.deliveryservice.docs.add_btn"
+22.Enter Name, type, document{randomAlpha} &gt;&gt; deliveryDocumentName, "admin.deliveryservice.docs.name_input"
+23.Open status Dropdown, click, , "admin.deliveryservice.docs.status_dropdown"
+24.Select Active, click, , "admin.deliveryservice.docs.status_option_active"
+25.Click Document Expiry, click, , "admin.deliveryservice.docs.expiry_checkbox"
+26.Click Document Expiry, click, , "admin.deliveryservice.docs.expiry_checkbox"
+27.Click Mandatory Document, click, , "admin.deliveryservice.docs.mandatory_checkbox"
+28.Click Require Proof Number, click, , "admin.deliveryservice.docs.proof_number_checkbox"
+29.Enter Display Order, type, 10, "admin.deliveryservice.docs.display_order_input"
+30.Click Submit, click, , "web.global.action.submit"
+31.Verify Success, verify, , "web.global.toast.info"
+32.Filter Document List, type, {deliveryDocumentName}, "admin.deliveryservice.docs.grid.filter_input"
+33.wait, 2000, , ""
+34.Click Settings, click, , "admin.deliveryservice.menu.toggle_btn"
+35.Click Promocode, click, , "admin.deliveryservice.submenu.promocode"
+36.Click Add Promo Code, click, , "admin.deliveryservice.promo.add_btn"
+37.Open User List Dropdown, click, , "admin.deliveryservice.promo.user_list_dropdown"
+38.Select User, click, , "admin.deliveryservice.promo.user_option_dynamic"
+39.Click Code Name Box, click, , "admin.deliveryservice.promo.code_name_box"
+40.Enter Code Name, type, promoCode{randomAlpha} &gt;&gt; deliveryPromoCodeName, "admin.deliveryservice.promo.code_name_box"
+41.Open Discount Type Dropdown, click, , "admin.deliveryservice.promo.discount_type_dropdown"
+42.Select Discount Type, click, , "admin.deliveryservice.promo.discount_type_option_amount"
+43.Enter Expiry Date, type, 12122026, "admin.deliveryservice.promo.expiry_date_input"
+44.Enter Discount Amount, type, 100, "admin.deliveryservice.promo.discount_amount_input"
+45.Enter Minimum Order Amount, type, 1000, "admin.deliveryservice.promo.min_order_input"
+46.Enter Maximum Discount Amount, type, 100, "admin.deliveryservice.promo.max_discount_input"
+47.Enter Coupon Limit, type, 5, "admin.deliveryservice.promo.coupon_limit_input"
+48.Enter Usage Limit for One User, type, 2, "admin.deliveryservice.promo.user_usage_limit_input"
+49.Enter Promo Code Description, type, Promo Code For Gold Member, "admin.deliveryservice.promo.description_textarea"
+50.Click Submit, click, , "web.global.action.submit"
+51.Verify Success, verify, , "web.global.toast.info"
+52.Filter PromoCode List, type, {deliveryPromoCodeName}, "admin.deliveryservice.promo.grid.filter_input"
+53.wait, 2000, , ""
+54.Click Settings, click, , "admin.deliveryservice.menu.toggle_btn"
+55.Click Service Settings, click, , "admin.deliveryservice.submenu.service_settings"
+56.Enter Driver Search Radius, type, 50, "admin.deliveryservice.config.search_radius_input"
+57.Open Tax Type Dropdown, click, , "admin.deliveryservice.config.tax_type_dropdown"
+58.Select Amount, click, , "admin.deliveryservice.config.tax_type_option_amount"
+59.Enter Tax, type, 20, "admin.deliveryservice.config.tax_input"
+60.Open Platform Fee Type Dropdown, click, , "admin.deliveryservice.config.fee_type_dropdown"
+61.Select Amount, click, , "admin.deliveryservice.config.fee_type_option_amount"
+62.Enter Platform Fee, type, 20, "admin.deliveryservice.config.platform_fee_input"
+63.Enter Cancel Charge (in %):, type, 20, "admin.deliveryservice.config.cancel_charge_input"
+64.Enter Driver Accept Timeout (in Second):, type, 20, "admin.deliveryservice.config.driver_timeout_input"
+65.Click Submit, click, , "web.global.action.submit"
+66.Verify Success, verify, , "web.global.toast.info"
+67.Click Stores, click, , "admin.store.menu.toggle_btn"
+68.Select Add Store, click, , "admin.store.submenu.add_store"
+69.Verify Add Store, verify, , "admin.store.add_page.header"
+70.Enter Store Name, type, amul_{timestamp} &gt;&gt; milkStore, "admin.store.name.input"
+71.Open Delivery Radius Dropdown, click, , "admin.store.radius.dropdown"
+72.Select Twenty Five Kilometer, click, , "admin.store.radius.option_25km"
+73.Open Estimated Delivery Time, click, , "admin.store.eta.dropdown"
+74.Select Thirty Minute, click, , "admin.store.eta.option_30min"
+75.Enter Order Minimum Amount, type, 300, "admin.store.min_amount.input"
+76.Enter Packaging Charges, type, 50, "admin.store.packaging_charge.input"
+77.Enter Short Description, type, amul taste of india, "admin.store.description.input"
+78.Upload Banner Image, uploadfile, "src/main/resources/test-data/amulbanner.jpg", "admin.store.banner.file"
+79.Open Driver Notification, click, , "admin.store.driver_notification.dropdown"
+80.Select Both Driver, click, , "admin.store.driver_notification.option_both"
+81.Click Checkbox Allow For Pickup, click, , "admin.store.allow_pickup.checkbox"
+82.Open Current Status Dropdown, click, , "admin.store.current_status.dropdown"
+83.Select Active, click, , "admin.store.current_status.option_active"
+84.Enter Store Address, type, Amul chennai, "admin.store.location.input"
+85.wait, 3000, , ""
+86.Confirm Store Address, press_enter, , "admin.store.location.input"
+87.wait, 3000, , ""
+88.Select First Option, arrow_down, , "admin.store.location.input"
+89.Confirm Option, press_enter, , "admin.store.location.input"
+90.wait, 2000, , ""
+91.Click Storewise Commission Checkbox, click, , "admin.store.commission.checkbox"
+92.Enter Store Commission, type, 25, "admin.store.commission_rate.input"
+93.Open Driver Notification, click, , "admin.store.offer_type.dropdown"
+94.Select Amount, click, , "admin.store.offer_type.option_amount"
+95.Enter Offer Amount, type, 50, "admin.store.offer_amount.input"
+96.Enter Offer Min Amount, type, 500, "admin.store.offer_min_amount.input"
+97.Enter Contact Person Full Name, type, amulStoreowner_{timestamp} &gt;&gt; milkStoreOwner, "admin.store.contact_name.input"
+98.Enter Email, type, amul_{timestamp}@gmail.com &gt;&gt; storeEmail, "admin.store.email.input"
+99.Enter Contact Number, type, {randomPhone}, "admin.store.phone.input"
+100.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "admin.store.profile.file"
+101.Enter Bank Name, type, federal, "admin.store.bank.name_input"
+102.Enter Bank Location, type, chennai, "admin.store.bank.location_input"
+103.Enter Account Number, type, 123456789012, "admin.store.bank.account_input"
+104.Enter Account Holder Name, type, {milkStoreOwner}, "admin.store.bank.holder_input"
+105.Enter Payment Email Address, type, {storeEmail}, "admin.store.bank.payment_email"
+106.Enter BIC Code, type, 1234, "admin.store.bank.bic_input"
+107.Click Store Timing Checkbox, click, , "admin.store.timing.everyday_checkbox"
+108.Enter From Time, type, 100000AM, "admin.store.timing.from_input"
+109.Enter To Time, type, 100000PM, "admin.store.timing.to_input"
+110.Submit Add Store, click, , "web.global.action.submit"
+111.Verify Success Message, verify, , "web.global.toast.info"
+112.Click Stores, click, , "admin.store.menu.toggle_btn"
+113.Select Store List, click, , "admin.store.submenu.store_list"
+114.Verify Add Store, verify, , "admin.store.list_page.header"
+115.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+116.Click Stores, click, , "admin.store.menu.toggle_btn"
+117.Select Pending Documents Stores List, click, , "admin.store.submenu.pending_docs"
+118.Verify Add Store, verify, , "admin.store.pending_page.header"
+119.Filter Pending Document Store List, type, {milkStore}, "admin.store.grid.name_filter"
+120.Scroll Grid, tab, 8, "admin.store.grid.name_filter"
+121.Click Doc Icon, click, , "admin.store.grid.doc_icon"
+122.Store Required Documents, verify, , "admin.store.documents_page.header"
+123.Add Address Proof, click, , "admin.store.grid.edit_doc_icon"
+124.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "admin.store.doc.file_input"
+125.Enter Expiry Date, type, 2026-12-12, "admin.store.doc.expiry_input"
+126.Click Submit, click, , "web.global.action.submit"
+127.Verify Updated Successfully, verify, , "web.global.toast.updated"
+128.Click Approve Store, click, , "admin.store.grid.approve_doc_icon"
+129.Verify Updated Successfully, verify, , "web.global.toast.updated"
+130.Click Back, click, , "admin.store.grid.back_btn"
+131.Click Stores, click, , "admin.store.menu.toggle_btn"
+132.Select Store List, click, , "admin.store.submenu.store_list"
+133.Verify Add Store, verify, , "admin.store.list_page.header"
+134.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+135.Scroll Grid, tab, 8, "admin.store.grid.name_filter"
+136.Click Doc Icon, click, , "admin.store.grid.doc_icon"
+137.Click Back, click, , "admin.store.grid.back_btn"
+138.Click Category, click, , "admin.deliveryservice.products.menu_category_btn"
+139.Click Add New Category, click, , "admin.deliveryservice.products.category.add_btn"
+140.Enter Category Name, type, curd{randomAlpha} &gt;&gt; MilkCategoryName, "admin.deliveryservice.products.category.name_input"
+141.Enter Category Name Arabic, type, رائب, "admin.deliveryservice.products.category.lang_arabic"
+142.Enter Category Name Tamil, type, தயிர், "admin.deliveryservice.products.category.lang_tamil"
+143.Enter Category Name Hindi, type, दही, "admin.deliveryservice.products.category.lang_hindi"
+144.Open Category status Dropdown, click, , "admin.deliveryservice.products.category.status_dropdown"
+145.Select Active, click, , "admin.deliveryservice.products.category.status_option_active"
+146.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "admin.deliveryservice.image.file"
+147.wait, 2000, , ""
+148.Enter Slug Name, type, curd, "admin.deliveryservice.products.category.slug_input"
+149.Click Submit, click, , "web.global.action.submit"
+150.Verify Success Message, verify, , "web.global.toast.info"
+151.Filter Category Name, type, {MilkCategoryName}, "admin.deliveryservice.products.category.grid.filter_input"
+152.Click Stores, click, , "admin.store.menu.toggle_btn"
+153.Select Store List, click, , "admin.store.submenu.store_list"
+154.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+155.Scroll Grid, tab, 9, "admin.store.grid.name_filter"
+156.Click Product Icon, click, , "admin.store.products.grid_icon"
+157.Click Add Products, click, , "admin.store.products.add_btn"
+158.Open Product Category Dropdown, click, , "admin.store.products.category_dropdown"
+159.Select curd, click, , "admin.deliveryservice.products.category.option_dynamic"
+160.wait, 1000, , ""
+161.Click badge, click, , "admin.store.badge.shield"
+162.Click Delivery Services, click, , "admin.store.delivery_services.menu"
+163.Verify Delivery Services, verify, , "admin.store.delivery_services.header"
+164.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+165.Click Edit Icon, click, , "admin.deliveryservice.grid.edit_icon"
+166.Open status Dropdown, click, , "admin.deliveryservice.status.dropdown"
+167.wait, 1000, , ""
+168.Select Deactivate, click, , "admin.deliveryservice.status.option_deactivate"
+169.Click Submit, click, , "web.global.action.submit"
+170.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+171.wait, 1000, , ""</t>
+  </si>
+  <si>
+    <t>Deleted Steps</t>
+  </si>
+  <si>
+    <t>34.Click Settings, click, , "admin.deliveryservice.menu.toggle_btn"
+35.Click Promocode, click, , "admin.deliveryservice.submenu.promocode"
+36.Click Add Promo Code, click, , "admin.deliveryservice.promo.add_btn"
+37.Open User List Dropdown, click, , "admin.deliveryservice.promo.user_list_dropdown"
+38.Select User, click, , "admin.deliveryservice.promo.user_option_dynamic"
+39.Click Code Name Box, click, , "admin.deliveryservice.promo.code_name_box"
+40.Enter Code Name, type, promoCode{randomAlpha} &gt;&gt; deliveryPromoCodeName, "admin.deliveryservice.promo.code_name_box"
+41.Open Discount Type Dropdown, click, , "admin.deliveryservice.promo.discount_type_dropdown"
+42.Select Discount Type, click, , "admin.deliveryservice.promo.discount_type_option_amount"
+43.Enter Expiry Date, type, 12122026, "admin.deliveryservice.promo.expiry_date_input"
+44.Enter Discount Amount, type, 100, "admin.deliveryservice.promo.discount_amount_input"
+45.Enter Minimum Order Amount, type, 1000, "admin.deliveryservice.promo.min_order_input"
+46.Enter Maximum Discount Amount, type, 100, "admin.deliveryservice.promo.max_discount_input"
+47.Enter Coupon Limit, type, 5, "admin.deliveryservice.promo.coupon_limit_input"
+48.Enter Usage Limit for One User, type, 2, "admin.deliveryservice.promo.user_usage_limit_input"
+49.Enter Promo Code Description, type, Promo Code For Gold Member, "admin.deliveryservice.promo.description_textarea"
+50.Click Submit, click, , "web.global.action.submit"
+51.Verify Success, verify, , "web.global.toast.info"
+52.Filter PromoCode List, type, {deliveryPromoCodeName}, "admin.deliveryservice.promo.grid.filter_input"
+53.wait, 2000, , ""</t>
+  </si>
+  <si>
+    <t>1.Click badge, click, , "admin.deliveryservice.badge.shield"
+2.Click Delivery Services, click, , "admin.deliveryservice.menu"
+3.Verify Delivery Services, verify, , "admin.deliveryservice.header"
+4.Click Add Service Category, click, , "admin.deliveryservice.add_category_btn"
+5.Enter Category Name, type, milk Delivery{randomAlpha} &gt;&gt; deliveryName, "admin.deliveryservice.category_name.input"
+6.Enter Slug, type, Milk Delivery, "admin.deliveryservice.slug.input"
+7.Upload Category Image, uploadfile, "src/main/resources/test-data/milkman.jpg", "admin.deliveryservice.image.file"
+8.Open status Dropdown, click, , "admin.deliveryservice.status.dropdown"
+9.Select Activate, click, , "admin.deliveryservice.status.option_activate"
+10.Open Category Flow Dropdown, click, , "admin.deliveryservice.flow.dropdown"
+11.Select default flow(food-delivery), click, , "admin.deliveryservice.flow.option_food_delivery"
+12.Enter Delivery Name Tamil, type, பால்காரர், "admin.deliveryservice.lang_tamil.input"
+13.Enter Delivery Name Arabic, type, لبّان, "admin.deliveryservice.lang_arabic.input"
+14.Enter Delivery Name Hindi, type, दूधवाला, "admin.deliveryservice.lang_hindi.input"
+15.Click Submit, click, , "web.global.action.submit"
+16.Verify Success, verify, , "web.global.toast.info"
+17.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+18.Click Home Icon, click, , "admin.deliveryservice.home.icon"
+19.Click Settings, click, , "admin.deliveryservice.settings.menu"
+20.Click Requirement Document, click, , "admin.deliveryservice.required_docs"
+21.Click Add Document, click, , "admin.deliveryservice.docs.add_btn"
+22.Enter Name, type, document{randomAlpha} &gt;&gt; deliveryDocumentName, "admin.deliveryservice.docs.name_input"
+23.Open status Dropdown, click, , "admin.deliveryservice.docs.status_dropdown"
+24.Select Active, click, , "admin.deliveryservice.docs.status_option_active"
+25.Click Document Expiry, click, , "admin.deliveryservice.docs.expiry_checkbox"
+26.Click Document Expiry, click, , "admin.deliveryservice.docs.expiry_checkbox"
+27.Click Mandatory Document, click, , "admin.deliveryservice.docs.mandatory_checkbox"
+28.Click Require Proof Number, click, , "admin.deliveryservice.docs.proof_number_checkbox"
+29.Enter Display Order, type, 10, "admin.deliveryservice.docs.display_order_input"
+30.Click Submit, click, , "web.global.action.submit"
+31.Verify Success, verify, , "web.global.toast.info"
+32.Filter Document List, type, {deliveryDocumentName}, "admin.deliveryservice.docs.grid.filter_input"
+33.wait, 2000, , ""
+34.Click Settings, click, , "admin.deliveryservice.settings.menu"
+35.Click Service Settings, click, , "admin.deliveryservice.submenu.service_settings"
+36.Enter Driver Search Radius, type, 50, "admin.deliveryservice.config.search_radius_input"
+37.Open Tax Type Dropdown, click, , "admin.deliveryservice.config.tax_type_dropdown"
+38.Select Amount, click, , "admin.deliveryservice.config.tax_type_option_amount"
+39.Enter Tax, type, 20, "admin.deliveryservice.config.tax_input"
+40.Open Platform Fee Type Dropdown, click, , "admin.deliveryservice.config.fee_type_dropdown"
+41.Select Amount, click, , "admin.deliveryservice.config.fee_type_option_amount"
+42.Enter Platform Fee, type, 20, "admin.deliveryservice.config.platform_fee_input"
+43.Enter Cancel Charge (in %):, type, 20, "admin.deliveryservice.config.cancel_charge_input"
+44.Enter Driver Accept Timeout (in Second):, type, 20, "admin.deliveryservice.config.driver_timeout_input"
+45.Click Submit, click, , "web.global.action.submit"
+46.Verify Success, verify, , "web.global.toast.info"
+47.Click Stores, click, , "admin.store.menu.toggle_btn"
+48.Select Add Store, click, , "admin.store.submenu.add_store"
+49.Verify Add Store, verify, , "admin.store.add_page.header"
+50.Enter Store Name, type, amul_{timestamp} &gt;&gt; milkStore, "admin.store.name.input"
+51.Open Delivery Radius Dropdown, click, , "admin.store.radius.dropdown"
+52.Select Twenty Five Kilometer, click, , "admin.store.radius.option_25km"
+53.Open Estimated Delivery Time, click, , "admin.store.eta.dropdown"
+54.Select Thirty Minute, click, , "admin.store.eta.option_30min"
+55.Enter Order Minimum Amount, type, 300, "admin.store.min_amount.input"
+56.Enter Packaging Charges, type, 50, "admin.store.packaging_charge.input"
+57.Enter Short Description, type, amul taste of india, "admin.store.description.input"
+58.Upload Banner Image, uploadfile, "src/main/resources/test-data/amulbanner.jpg", "admin.store.banner.file"
+59.Open Driver Notification, click, , "admin.store.driver_notification.dropdown"
+60.Select Both Driver, click, , "admin.store.driver_notification.option_both"
+61.Click Checkbox Allow For Pickup, click, , "admin.store.allow_pickup.checkbox"
+62.Open Current Status Dropdown, click, , "admin.store.current_status.dropdown"
+63.Select Active, click, , "admin.store.current_status.option_active"
+64.Enter Store Address, type, Amul chennai, "admin.store.location.input"
+65.wait, 3000, , ""
+66.Confirm Store Address, press_enter, , "admin.store.location.input"
+67.wait, 3000, , ""
+68.Select First Option, arrow_down, , "admin.store.location.input"
+69.Confirm Option, press_enter, , "admin.store.location.input"
+70.wait, 2000, , ""
+71.Click Storewise Commission Checkbox, click, , "admin.store.commission.checkbox"
+72.Enter Store Commission, type, 25, "admin.store.commission_rate.input"
+73.Open Driver Notification, click, , "admin.store.offer_type.dropdown"
+74.Select Amount, click, , "admin.store.offer_type.option_amount"
+75.Enter Offer Amount, type, 50, "admin.store.offer_amount.input"
+76.Enter Offer Min Amount, type, 500, "admin.store.offer_min_amount.input"
+77.Enter Contact Person Full Name, type, amulStoreowner_{timestamp} &gt;&gt; milkStoreOwner, "admin.store.contact_name.input"
+78.Enter Email, type, amul_{timestamp}@gmail.com &gt;&gt; storeEmail, "admin.store.email.input"
+79.Enter Contact Number, type, {randomPhone}, "admin.store.phone.input"
+80.Upload Store Image, uploadfile, "src/main/resources/test-data/milkbooth.jpeg", "admin.store.profile.file"
+81.Enter Bank Name, type, federal, "admin.store.bank.name_input"
+82.Enter Bank Location, type, chennai, "admin.store.bank.location_input"
+83.Enter Account Number, type, 123456789012, "admin.store.bank.account_input"
+84.Enter Account Holder Name, type, {milkStoreOwner}, "admin.store.bank.holder_input"
+85.Enter Payment Email Address, type, {storeEmail}, "admin.store.bank.payment_email"
+86.Enter BIC Code, type, 1234, "admin.store.bank.bic_input"
+87.Click Store Timing Checkbox, click, , "admin.store.timing.everyday_checkbox"
+88.Enter From Time, type, 100000AM, "admin.store.timing.from_input"
+89.Enter To Time, type, 100000PM, "admin.store.timing.to_input"
+90.Submit Add Store, click, , "web.global.action.submit"
+91.Verify Success Message, verify, , "web.global.toast.info"
+92.Click Stores, click, , "admin.store.menu.toggle_btn"
+93.Select Store List, click, , "admin.store.submenu.store_list"
+94.Verify Add Store, verify, , "admin.store.list_page.header"
+95.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+96.Click Stores, click, , "admin.store.menu.toggle_btn"
+97.Select Pending Documents Stores List, click, , "admin.store.submenu.pending_docs"
+98.Verify Add Store, verify, , "admin.store.pending_page.header"
+99.Filter Pending Document Store List, type, {milkStore}, "admin.store.grid.name_filter"
+100.Scroll Grid, tab, 8, "admin.store.grid.name_filter"
+101.Click Doc Icon, click, , "admin.store.grid.doc_icon"
+102.Store Required Documents, verify, , "admin.store.documents_page.header"
+103.Add Address Proof, click, , "admin.store.grid.edit_doc_icon"
+104.Upload Address Proof, uploadfile, "src/main/resources/test-data/addressproof.png", "admin.store.doc.file_input"
+105.Enter Expiry Date, type, 2026-12-12, "admin.store.doc.expiry_input"
+106.Click Submit, click, , "web.global.action.submit"
+107.Verify Updated Successfully, verify, , "web.global.toast.updated"
+108.Click Approve Store, click, , "admin.store.grid.approve_doc_icon"
+109.Verify Updated Successfully, verify, , "web.global.toast.updated"
+110.Click Back, click, , "admin.store.grid.back_btn"
+111.Click Stores, click, , "admin.store.menu.toggle_btn"
+112.Select Store List, click, , "admin.store.submenu.store_list"
+113.Verify Add Store, verify, , "admin.store.list_page.header"
+114.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+115.Scroll Grid, tab, 8, "admin.store.grid.name_filter"
+116.Click Doc Icon, click, , "admin.store.grid.doc_icon"
+117.Click Back, click, , "admin.store.grid.back_btn"
+118.Click Category, click, , "admin.deliveryservice.products.menu_category_btn"
+119.Click Add New Category, click, , "admin.deliveryservice.products.category.add_btn"
+120.Enter Category Name, type, curd{randomAlpha} &gt;&gt; MilkCategoryName, "admin.deliveryservice.products.category.name_input"
+121.Enter Category Name Arabic, type, رائب, "admin.deliveryservice.products.category.lang_arabic"
+122.Enter Category Name Tamil, type, தயிர், "admin.deliveryservice.products.category.lang_tamil"
+123.Enter Category Name Hindi, type, दही, "admin.deliveryservice.products.category.lang_hindi"
+124.Open Category status Dropdown, click, , "admin.deliveryservice.products.category.status_dropdown"
+125.Select Active, click, , "admin.deliveryservice.products.category.status_option_active"
+126.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "admin.deliveryservice.image.file"
+127.wait, 2000, , ""
+128.Enter Slug Name, type, curd, "admin.deliveryservice.products.category.slug_input"
+129.Click Submit, click, , "web.global.action.submit"
+130.Verify Success Message, verify, , "web.global.toast.info"
+131.Filter Category Name, type, {MilkCategoryName}, "admin.deliveryservice.products.category.grid.filter_input"
+132.Click Stores, click, , "admin.store.menu.toggle_btn"
+133.Select Store List, click, , "admin.store.submenu.store_list"
+134.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+135.Scroll Grid, tab, 9, "admin.store.grid.name_filter"
+136.Click Product Icon, click, , "admin.store.products.grid_icon"
+137.Click Add Products, click, , "admin.store.products.add_btn"
+138.Open Product Category Dropdown, click, , "admin.store.products.category_dropdown"
+139.Select curd, click, , "admin.deliveryservice.products.category.option_dynamic"
+140.wait, 1000, ,""
+141.Click badge, click, , "admin.deliveryservice.badge.shield"
+142.Click Delivery Services, click, , "admin.deliveryservice.menu"
+143.Verify Delivery Services, verify, , "admin.deliveryservice.header"
+144.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+145.Click Edit Icon, click, , "admin.deliveryservice.grid.edit_icon"
+146.Open status Dropdown, click, , "admin.deliveryservice.status.dropdown"
+147.wait, 1000, , ""
+148.Select Deactivate, click, , "admin.deliveryservice.status.option_deactivate"
+149.Click Submit, click, , "web.global.action.submit"
+150.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+151.wait, 1000, ,</t>
+  </si>
+  <si>
+    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+2. Click Delivery Services,click,,"admin.deliveryservice.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
 4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
 5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
 6. Click Stores,click,,"admin.store.menu.toggle_btn"
@@ -2900,79 +3153,9 @@
 77. wait,1000,,</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Data Dependency: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The AddStore test suite must be always executed before this test. This is critical because the StoreOperations process utilizes the dynamic {storeName} variable generated and stored during the AddStore creation phase.
-RunSheet: AddStore2
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Authentication State: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">The user is already authenticated as a Super Admin and the session is active.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Navigation State:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The browser is currently on the Dashboard page. Ensure the dashboard.url is configured as https://dev.we1.co/#/page-module/dashboard_dynamic in the config.properties file.
-</t>
-    </r>
-  </si>
-  <si>
-    <t>1. Click badge,click,,"admin.store.badge.shield"
-2. Click Delivery Services,click,,"admin.store.delivery_services.menu"
-3. Wait For Delivery Services,wait_until_visible,,"admin.store.delivery_services.header"
+    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+2. Click Delivery Services,click,,"admin.deliveryservice.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
 4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
 5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
 6. Click Stores,click,,"admin.store.menu.toggle_btn"
@@ -3037,9 +3220,9 @@
 65. wait,1000,,</t>
   </si>
   <si>
-    <t>1. Click badge,click,,"admin.store.badge.shield"
-2. Click Delivery Services,click,,"admin.store.delivery_services.menu"
-3. Wait For Delivery Services,wait_until_visible,,"admin.store.delivery_services.header"
+    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+2. Click Delivery Services,click,,"admin.deliveryservice.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
 4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
 5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
 6. Click Stores,click,,"admin.store.menu.toggle_btn"
@@ -3559,7 +3742,7 @@
         <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>37</v>
@@ -3628,13 +3811,13 @@
         <v>27</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -3700,16 +3883,16 @@
         <v>30</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3772,13 +3955,13 @@
         <v>32</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -3797,7 +3980,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73960651-1493-478A-BEDA-A31CF297E315}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8A1C6E6-1358-42F0-B7B3-06420689DEE4}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3807,7 +3990,8 @@
     <col min="4" max="4" width="34.109375" customWidth="1"/>
     <col min="5" max="5" width="69.33203125" customWidth="1"/>
     <col min="6" max="6" width="31.77734375" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" customWidth="1"/>
+    <col min="7" max="7" width="44.33203125" customWidth="1"/>
+    <col min="8" max="8" width="27.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -3830,10 +4014,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>6</v>
+        <v>112</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>7</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
@@ -3844,16 +4028,22 @@
         <v>54</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>57</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>74</v>
+        <v>116</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>58</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -3916,7 +4106,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>36</v>
@@ -3988,7 +4178,7 @@
         <v>40</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>56</v>
@@ -4060,13 +4250,13 @@
         <v>69</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>72</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>71</v>
@@ -4126,19 +4316,19 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>65</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>66</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>67</v>
@@ -4193,7 +4383,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4213,13 +4403,13 @@
         <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4292,7 +4482,7 @@
         <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>41</v>
@@ -4347,7 +4537,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4367,13 +4557,13 @@
         <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>38</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -4415,7 +4605,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4429,19 +4619,19 @@
         <v>14</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>42</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4490,7 +4680,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4504,19 +4694,19 @@
         <v>15</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>43</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4565,7 +4755,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4579,19 +4769,19 @@
         <v>17</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>44</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4640,7 +4830,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>7</v>
@@ -4654,19 +4844,19 @@
         <v>60</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>63</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>62</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4724,22 +4914,22 @@
     </row>
     <row r="2" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="D2" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
73th Commit: Keyword Refernce File Updated For Excel Test Step Explanation
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32BF513C-6185-45BE-8062-0F8880287EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC13A97E-358D-43E7-AB26-196297D4DAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2921,6 +2921,251 @@
 53.wait, 2000, , ""</t>
   </si>
   <si>
+    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+2. Click Delivery Services,click,,"admin.deliveryservice.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
+4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
+5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
+6. Click Stores,click,,"admin.store.menu.toggle_btn"
+7. Select Add Store,click,,"admin.store.submenu.add_store"
+8. Wait For Add Store,wait_until_visible,,"admin.store.add_page.header"
+9. Enter Store Name,type,KFC_{timestamp} &gt;&gt; storeName,"admin.store.name.input"
+10. Open Delivery Radius Dropdown,click,,"admin.store.radius.dropdown"
+11. Select Twenty Five Kilometer,click,,"admin.store.radius.option_25km"
+12. Open Estimated Delivery Time,click,,"admin.store.eta.dropdown"
+13. Select Thirty Minute,click,,"admin.store.eta.option_30min"
+14. Enter Order Minimum Amount,type,300,"admin.store.min_amount.input"
+15. Enter Packaging Charges,type,50,"admin.store.packaging_charge.input"
+16. Enter Short Description,type,KFC is a global fast-food giant famous for its Original Recipe fried chicken,"admin.store.description.input"
+17. Upload Banner Image,uploadfile,"src/main/resources/test-data/kfcbanner.jpg","admin.store.banner.file"
+18. Open Driver Notification,click,,"admin.store.driver_notification.dropdown"
+19. Select Both Driver,click,,"admin.store.driver_notification.option_both"
+20. Click Checkbox Allow For Pickup,click,,"admin.store.allow_pickup.checkbox"
+21. Open Current Status Dropdown,click,,"admin.store.current_status.dropdown"
+22. Select Active,click,,"admin.store.current_status.option_active"
+23. Enter Store Address,type,KFC chennai,"admin.store.location.input"
+24. wait,3000,,
+25. Confirm Store Address,press_enter,,"admin.store.location.input"
+26. wait,3000,,
+27. Select First Option,arrow_down,,"admin.store.location.input"
+28. Confirm Option,press_enter,,"admin.store.location.input"
+29. wait,2000,,
+30. Click Storewise Comission Checkbox,click,,"admin.store.commission.checkbox"
+31. Enter Store Commision,type,25,"admin.store.commission_rate.input"
+32. Open Driver Notification,click,,"admin.store.offer_type.dropdown"
+33. Select Amount,click,,"admin.store.offer_type.option_amount"
+34. Enter Offer Amount,type,50,"admin.store.offer_amount.input"
+35. Enter Offer Min Amount,type,500,"admin.store.offer_min_amount.input"
+36. Enter Contact Person Full Name,type,storeowner_{timestamp} &gt;&gt; storeOwner,"admin.store.contact_name.input"
+37. Enter Email,type,kfc_{timestamp}@gmail.com&gt;&gt;storeEmail,"admin.store.email.input"
+38. Enter Contact Number,type,{randomPhone},"admin.store.phone.input"
+39. Upload Store Image,uploadfile,"src/main/resources/test-data/kfcstore.jpg","admin.store.profile.file"
+40. Enter Bank Name,type,federal,"admin.store.bank.name_input"
+41. Enter Bank Location,type,chennai,"admin.store.bank.location_input"
+42. Enter Account Number,type,123456789012,"admin.store.bank.account_input"
+43. Enter Accont Holder Name,type,{storeOwner},"admin.store.bank.holder_input"
+44. Enter Payment Email Address,type,{storeEmail},"admin.store.bank.payment_email"
+45. Enter BIC Code,type,1234,"admin.store.bank.bic_input"
+46. Click Store Timing Checkbox,click,,"admin.store.timing.everyday_checkbox"
+47. Enter From Time,type,100000AM,"admin.store.timing.from_input"
+48. Enter To Time,type,100000PM,"admin.store.timing.to_input"
+49. Submit Add Store,click,,"web.global.action.submit"
+50. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
+51. Click Stores,click,,"admin.store.menu.toggle_btn"
+52. Select Store List,click,,"admin.store.submenu.store_list"
+53. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+54. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+55. Click Stores,click,,"admin.store.menu.toggle_btn"
+56. Select Pending Documents Stores List,click,,"admin.store.submenu.pending_docs"
+57. Wait For Add Store,wait_until_visible,,"admin.store.pending_page.header"
+58. Filter Pending Document Store List,type,{storeName},"admin.store.grid.name_filter"
+59. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+60. Click Doc Icon,click,,"admin.store.grid.doc_icon"
+61. Store Required Documents,verify,,"admin.store.documents_page.header"
+62. Add Address Proof,click,,"admin.store.grid.edit_doc_icon"
+63. Upload Address Proof,uploadfile,"src/main/resources/test-data/addressproof.png","admin.store.doc.file_input"
+64. Enter Expiry Date,type,2026-12-12,"admin.store.doc.expiry_input"
+65. Click Submit,click,,"web.global.action.submit"
+66. Verify Updated Succesfully,verify,,"web.global.toast.updated"
+67. Click Approve Store,click,,"admin.store.grid.approve_doc_icon"
+68. Verify Updated Succesfully,verify,,"web.global.toast.updated"
+69. Click Back,click,,"admin.store.grid.back_btn"
+70. Click Stores,click,,"admin.store.menu.toggle_btn"
+71. Select Store List,click,,"admin.store.submenu.store_list"
+72. Verify Add Store,verify,,"admin.store.list_page.header"
+73. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+74. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+75. Click Doc Icon,click,,"admin.store.grid.doc_icon"
+76. Click Eye Icon,click,,"admin.store.grid.eye_view_icon"
+77. wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+2. Click Delivery Services,click,,"admin.deliveryservice.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
+4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
+5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
+6. Click Stores,click,,"admin.store.menu.toggle_btn"
+7. Select Store List,click,,"admin.store.submenu.store_list"
+8. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+9. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+10. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+11. Click Product Icon,click,,"admin.store.products.grid_icon"
+12. Click Add Products,click,,"admin.store.products.add_btn"
+13. Open Product Category Dropdown,click,,"admin.store.products.category_dropdown"
+14. Select Grill Chicken,click,,"admin.store.products.category_option_grill"
+15. Enter Product Name,type,kfcProduct{randomAlpha}&gt;&gt; kfcProductName,"admin.store.products.name_input"
+16. Enter Product Amount,type,500,"admin.store.products.amount_input"
+17. Enter Product Description,type,KFC special grill chicken,"admin.store.products.description_textarea"
+18. Upload Product Image,uploadfile,"src/main/resources/test-data/grillchicken.jpg","admin.store.products.image.file"
+19. Open Product Category Dropdown,click,,"admin.store.products.status_dropdown"
+20. Select Activate,click,,"admin.store.products.status_option_active"
+21. Open Discount Type Dropdown,click,,"admin.store.products.discount_dropdown"
+22. Enter Discount Amount,type,50,"admin.store.products.discount_input"
+23. Click Save,click,,"admin.store.products.save_btn"
+24. Wait For Saved Succesfully,wait_until_visible,,"admin.store.products.toast_success"
+25. Wait For Store Products,wait_until_visible,,"admin.store.products.header"
+26. Filter Product List,type,{kfcProductName},"admin.store.products.name_filter"
+27. Click Back,click,,"admin.store.products.back_btn"
+28. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+29. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+30. Click Wallet Icon,click,,"admin.store.wallet.grid_icon"
+31. Click Manage Transaction,click,,"admin.store.wallet.manage_transaction_btn"
+32. Enter Wallet Amount,type,1000,"admin.store.wallet.amount_input"
+33. Open Choose Option Dropdown,click,,"admin.store.wallet.option_dropdown"
+34. Select Add Money,click,,"admin.store.wallet.option_add"
+35. Click Submit,click,,"web.global.action.submit"
+36. Wait For Saved Succesfully,wait_until_visible,,"web.global.toast.success"
+37. Click Manage Transaction,click,,"admin.store.wallet.manage_transaction_btn"
+38. Enter Wallet Amount,type,200,"admin.store.wallet.amount_input"
+39. Open Choose Option Dropdown,click,,"admin.store.wallet.option_dropdown"
+40. Select Deduct Money,click,,"admin.store.wallet.option_deduct"
+41. Click Submit,click,,"web.global.action.submit"
+42. Wait For Saved Succesfully,wait_until_visible,,"web.global.toast.success"
+43. Click Back,click,,"admin.store.products.back_btn"
+44. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
+45. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+46. Click Drivers Icon,click,,"admin.store.drivers.grid_icon"
+47. Click Add Private Driver,click,,"admin.store.drivers.add_private_btn"
+48. Enter Driver Name,type,kfcdriver_{timestamp} &gt;&gt; kfcdriverName,"admin.drivers.fullname.input"
+49. Enter Email,type,kfcdriver_{timestamp}@gmail.com,"admin.drivers.email.input"
+50. Enter Contact Number,type,{randomPhone},"admin.drivers.phone.input"
+51. Upload Profile Image,uploadfile,"src/main/resources/test-data/bikedriver.jpg","admin.drivers.profile_image.file"
+52. Select Male Gender,click,,"admin.drivers.male_gender.div"
+53. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+54. Select Scooter Option,click,,"admin.drivers.vehicle_option.scooter"
+55. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
+56. Enter Vehicle Company,type,kfcBikeCompany{randomAlpha}&gt;&gt; kfcBikeCompanyName,"admin.drivers.companyname.input"
+57. Enter Plate No,type,KL-01-AB-1634,"admin.drivers.plateno.input"
+58. Enter Model Name,type,activa,"admin.drivers.modelname.input"
+59. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/bike.jpg","admin.drivers.vehicle_image.file"
+60. Enter Vehicle Color,type,white,"admin.drivers.vehicle_color.input"
+61. Click Submit,click,,"web.global.action.submit"
+62. Wait For Driver Added,wait_until_visible,,"web.global.toast.success"
+63. Filter Driver List,type,{kfcdriverName},"admin.drivers.name_filter.input"
+64. Click Eye Icon,click,,"admin.store.grid.eye_view_icon"
+65. wait,1000,,</t>
+  </si>
+  <si>
+    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
+2. Click Delivery Services,click,,"admin.deliveryservice.menu"
+3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
+4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
+5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
+6. Click Stores,click,,"admin.store.menu.toggle_btn"
+7. Select Add Store,click,,"admin.store.submenu.add_store"
+8. Wait For Add Store,wait_until_visible,,"admin.store.add_page.header"
+9. Enter Store Name,type,bilal_{timestamp} &gt;&gt; hotelName,"admin.store.name.input"
+10. Open Delivery Radius Dropdown,click,,"admin.store.radius.dropdown"
+11. Select Twenty Five Kilometer,click,,"admin.store.radius.option_25km"
+12. Open Estimated Delivery Time,click,,"admin.store.eta.dropdown"
+13. Select Thirty Minute,click,,"admin.store.eta.option_30min"
+14. Enter Order Minimum Amount,type,300,"admin.store.min_amount.input"
+15. Enter Packaging Charges,type,50,"admin.store.packaging_charge.input"
+16. Enter Short Description,type,KFC is a global fast-food giant famous for its Original Recipe fried chicken,"admin.store.description.input"
+17. Upload Banner Image,uploadfile,"src/main/resources/test-data/kfcbanner.jpg","admin.store.banner.file"
+18. Open Driver Notification,click,,"admin.store.driver_notification.dropdown"
+19. Select Both Driver,click,,"admin.store.driver_notification.option_both"
+20. Click Checkbox Allow For Pickup,click,,"admin.store.allow_pickup.checkbox"
+21. Open Current Status Dropdown,click,,"admin.store.current_status.dropdown"
+22. Select Active,click,,"admin.store.current_status.option_active"
+23. Enter Store Address,type,KFC chennai,"admin.store.location.input"
+24. wait,3000,,
+25. Confirm Store Address,press_enter,,"admin.store.location.input"
+26. wait,3000,,
+27. Select First Option,arrow_down,,"admin.store.location.input"
+28. Confirm Option,press_enter,,"admin.store.location.input"
+29. wait,2000,,
+30. Click Storewise Comission Checkbox,click,,"admin.store.commission.checkbox"
+31. Enter Store Commision,type,25,"admin.store.commission_rate.input"
+32. Open Driver Notification,click,,"admin.store.offer_type.dropdown"
+33. Select Amount,click,,"admin.store.offer_type.option_amount"
+34. Enter Offer Amount,type,50,"admin.store.offer_amount.input"
+35. Enter Offer Min Amount,type,500,"admin.store.offer_min_amount.input"
+36. Enter Contact Person Full Name,type,bilalowner_{timestamp} &gt;&gt; hotelOwner,"admin.store.contact_name.input"
+37. Enter Email,type,bilal_{timestamp}@gmail.com&gt;&gt;storeEmail,"admin.store.email.input"
+38. Enter Contact Number,type,{randomPhone},"admin.store.phone.input"
+39. Upload Store Image,uploadfile,"src/main/resources/test-data/kfcstore.jpg","admin.store.profile.file"
+40. Enter Bank Name,type,federal,"admin.store.bank.name_input"
+41. Enter Bank Location,type,chennai,"admin.store.bank.location_input"
+42. Enter Account Number,type,123456789012,"admin.store.bank.account_input"
+43. Enter Accont Holder Name,type,{hotelOwner},"admin.store.bank.holder_input"
+44. Enter Payment Email Address,type,{storeEmail},"admin.store.bank.payment_email"
+45. Enter BIC Code,type,1234,"admin.store.bank.bic_input"
+46. Click Store Timing Checkbox,click,,"admin.store.timing.everyday_checkbox"
+47. Enter From Time,type,100000AM,"admin.store.timing.from_input"
+48. Enter To Time,type,100000PM,"admin.store.timing.to_input"
+49. Submit Add Store,click,,"web.global.action.submit"
+50. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
+51. Click Stores,click,,"admin.store.menu.toggle_btn"
+52. Select Store List,click,,"admin.store.submenu.store_list"
+53. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+54. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+55. Click Stores,click,,"admin.store.menu.toggle_btn"
+56. Select Pending Documents Stores List,click,,"admin.store.submenu.pending_docs"
+57. Wait For Add Store,wait_until_visible,,"admin.store.pending_page.header"
+58. Filter Pending Document Store List,type,{hotelName},"admin.store.grid.name_filter"
+59. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+60. Click Doc Icon,click,,"admin.store.grid.doc_icon"
+61. Wait For Store Required Documents,wait_until_visible,,"admin.store.documents_page.header"
+62. Add Address Proof,click,,"admin.store.grid.edit_doc_icon"
+63. Upload Address Proof,uploadfile,"src/main/resources/test-data/addressproof.png","admin.store.doc.file_input"
+64. Enter Expiry Date,type,2026-12-12,"admin.store.doc.expiry_input"
+65. Click Submit,click,,"web.global.action.submit"
+66. Wait For Updated Succesfully,wait_until_visible,,"web.global.toast.updated"
+67. Click Approve Store,click,,"admin.store.grid.approve_doc_icon"
+68. Verify Updated Succesfully,verify,,"web.global.toast.updated"
+69. Click Back,click,,"admin.store.grid.back_btn"
+70. Click Stores,click,,"admin.store.menu.toggle_btn"
+71. Select Store List,click,,"admin.store.submenu.store_list"
+72. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
+73. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+74. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+75. Click Block Icon,click,,"admin.store.grid.block_icon"
+76. Click Block Yes,click,,"web.global.dialog.btn_confirm_yes"
+77. Click Stores,click,,"admin.store.menu.toggle_btn"
+78. Select Blocked Store,click,,"admin.store.submenu.blocked_stores"
+79. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+80. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+81. Click unBlock Icon,click,,"admin.store.grid.unblock_icon"
+82. Click Stores,click,,"admin.store.menu.toggle_btn"
+83. Select Rejected Store,click,,"admin.store.submenu.rejected_stores"
+84. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+85. Scroll Grid,tab,7,"admin.store.grid.name_filter"
+86. Click Approve Icon,click,,"admin.store.grid.approve_icon"
+87. Click Stores,click,,"admin.store.menu.toggle_btn"
+88. Select Store List,click,,"admin.store.submenu.store_list"
+89. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
+90. wait,3000,,
+91. Scroll Grid,tab,8,"admin.store.grid.name_filter"
+92. Click Doc Icon,click,,"admin.store.grid.document_icon"
+93. Click UnApprove Icon,click,,"admin.store.grid.unapprove_icon"
+94. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
+95. Rejection Reason,type,document insufficent,"web.global.dialog.textarea_reason"
+96. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
+97. wait,1000,,</t>
+  </si>
+  <si>
     <t>1.Click badge, click, , "admin.deliveryservice.badge.shield"
 2.Click Delivery Services, click, , "admin.deliveryservice.menu"
 3.Verify Delivery Services, verify, , "admin.deliveryservice.header"
@@ -3037,286 +3282,42 @@
 114.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
 115.Scroll Grid, tab, 8, "admin.store.grid.name_filter"
 116.Click Doc Icon, click, , "admin.store.grid.doc_icon"
-117.Click Back, click, , "admin.store.grid.back_btn"
-118.Click Category, click, , "admin.deliveryservice.products.menu_category_btn"
-119.Click Add New Category, click, , "admin.deliveryservice.products.category.add_btn"
-120.Enter Category Name, type, curd{randomAlpha} &gt;&gt; MilkCategoryName, "admin.deliveryservice.products.category.name_input"
-121.Enter Category Name Arabic, type, رائب, "admin.deliveryservice.products.category.lang_arabic"
-122.Enter Category Name Tamil, type, தயிர், "admin.deliveryservice.products.category.lang_tamil"
-123.Enter Category Name Hindi, type, दही, "admin.deliveryservice.products.category.lang_hindi"
-124.Open Category status Dropdown, click, , "admin.deliveryservice.products.category.status_dropdown"
-125.Select Active, click, , "admin.deliveryservice.products.category.status_option_active"
-126.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "admin.deliveryservice.image.file"
-127.wait, 2000, , ""
-128.Enter Slug Name, type, curd, "admin.deliveryservice.products.category.slug_input"
-129.Click Submit, click, , "web.global.action.submit"
-130.Verify Success Message, verify, , "web.global.toast.info"
-131.Filter Category Name, type, {MilkCategoryName}, "admin.deliveryservice.products.category.grid.filter_input"
-132.Click Stores, click, , "admin.store.menu.toggle_btn"
-133.Select Store List, click, , "admin.store.submenu.store_list"
-134.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
-135.Scroll Grid, tab, 9, "admin.store.grid.name_filter"
-136.Click Product Icon, click, , "admin.store.products.grid_icon"
-137.Click Add Products, click, , "admin.store.products.add_btn"
-138.Open Product Category Dropdown, click, , "admin.store.products.category_dropdown"
-139.Select curd, click, , "admin.deliveryservice.products.category.option_dynamic"
-140.wait, 1000, ,""
-141.Click badge, click, , "admin.deliveryservice.badge.shield"
-142.Click Delivery Services, click, , "admin.deliveryservice.menu"
-143.Verify Delivery Services, verify, , "admin.deliveryservice.header"
-144.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
-145.Click Edit Icon, click, , "admin.deliveryservice.grid.edit_icon"
-146.Open status Dropdown, click, , "admin.deliveryservice.status.dropdown"
-147.wait, 1000, , ""
-148.Select Deactivate, click, , "admin.deliveryservice.status.option_deactivate"
-149.Click Submit, click, , "web.global.action.submit"
-150.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
-151.wait, 1000, ,</t>
-  </si>
-  <si>
-    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
-2. Click Delivery Services,click,,"admin.deliveryservice.menu"
-3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
-4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
-5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
-6. Click Stores,click,,"admin.store.menu.toggle_btn"
-7. Select Add Store,click,,"admin.store.submenu.add_store"
-8. Wait For Add Store,wait_until_visible,,"admin.store.add_page.header"
-9. Enter Store Name,type,KFC_{timestamp} &gt;&gt; storeName,"admin.store.name.input"
-10. Open Delivery Radius Dropdown,click,,"admin.store.radius.dropdown"
-11. Select Twenty Five Kilometer,click,,"admin.store.radius.option_25km"
-12. Open Estimated Delivery Time,click,,"admin.store.eta.dropdown"
-13. Select Thirty Minute,click,,"admin.store.eta.option_30min"
-14. Enter Order Minimum Amount,type,300,"admin.store.min_amount.input"
-15. Enter Packaging Charges,type,50,"admin.store.packaging_charge.input"
-16. Enter Short Description,type,KFC is a global fast-food giant famous for its Original Recipe fried chicken,"admin.store.description.input"
-17. Upload Banner Image,uploadfile,"src/main/resources/test-data/kfcbanner.jpg","admin.store.banner.file"
-18. Open Driver Notification,click,,"admin.store.driver_notification.dropdown"
-19. Select Both Driver,click,,"admin.store.driver_notification.option_both"
-20. Click Checkbox Allow For Pickup,click,,"admin.store.allow_pickup.checkbox"
-21. Open Current Status Dropdown,click,,"admin.store.current_status.dropdown"
-22. Select Active,click,,"admin.store.current_status.option_active"
-23. Enter Store Address,type,KFC chennai,"admin.store.location.input"
-24. wait,3000,,
-25. Confirm Store Address,press_enter,,"admin.store.location.input"
-26. wait,3000,,
-27. Select First Option,arrow_down,,"admin.store.location.input"
-28. Confirm Option,press_enter,,"admin.store.location.input"
-29. wait,2000,,
-30. Click Storewise Comission Checkbox,click,,"admin.store.commission.checkbox"
-31. Enter Store Commision,type,25,"admin.store.commission_rate.input"
-32. Open Driver Notification,click,,"admin.store.offer_type.dropdown"
-33. Select Amount,click,,"admin.store.offer_type.option_amount"
-34. Enter Offer Amount,type,50,"admin.store.offer_amount.input"
-35. Enter Offer Min Amount,type,500,"admin.store.offer_min_amount.input"
-36. Enter Contact Person Full Name,type,storeowner_{timestamp} &gt;&gt; storeOwner,"admin.store.contact_name.input"
-37. Enter Email,type,kfc_{timestamp}@gmail.com&gt;&gt;storeEmail,"admin.store.email.input"
-38. Enter Contact Number,type,{randomPhone},"admin.store.phone.input"
-39. Upload Store Image,uploadfile,"src/main/resources/test-data/kfcstore.jpg","admin.store.profile.file"
-40. Enter Bank Name,type,federal,"admin.store.bank.name_input"
-41. Enter Bank Location,type,chennai,"admin.store.bank.location_input"
-42. Enter Account Number,type,123456789012,"admin.store.bank.account_input"
-43. Enter Accont Holder Name,type,{storeOwner},"admin.store.bank.holder_input"
-44. Enter Payment Email Address,type,{storeEmail},"admin.store.bank.payment_email"
-45. Enter BIC Code,type,1234,"admin.store.bank.bic_input"
-46. Click Store Timing Checkbox,click,,"admin.store.timing.everyday_checkbox"
-47. Enter From Time,type,100000AM,"admin.store.timing.from_input"
-48. Enter To Time,type,100000PM,"admin.store.timing.to_input"
-49. Submit Add Store,click,,"web.global.action.submit"
-50. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
-51. Click Stores,click,,"admin.store.menu.toggle_btn"
-52. Select Store List,click,,"admin.store.submenu.store_list"
-53. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
-54. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
-55. Click Stores,click,,"admin.store.menu.toggle_btn"
-56. Select Pending Documents Stores List,click,,"admin.store.submenu.pending_docs"
-57. Wait For Add Store,wait_until_visible,,"admin.store.pending_page.header"
-58. Filter Pending Document Store List,type,{storeName},"admin.store.grid.name_filter"
-59. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-60. Click Doc Icon,click,,"admin.store.grid.doc_icon"
-61. Store Required Documents,verify,,"admin.store.documents_page.header"
-62. Add Address Proof,click,,"admin.store.grid.edit_doc_icon"
-63. Upload Address Proof,uploadfile,"src/main/resources/test-data/addressproof.png","admin.store.doc.file_input"
-64. Enter Expiry Date,type,2026-12-12,"admin.store.doc.expiry_input"
-65. Click Submit,click,,"web.global.action.submit"
-66. Verify Updated Succesfully,verify,,"web.global.toast.updated"
-67. Click Approve Store,click,,"admin.store.grid.approve_doc_icon"
-68. Verify Updated Succesfully,verify,,"web.global.toast.updated"
-69. Click Back,click,,"admin.store.grid.back_btn"
-70. Click Stores,click,,"admin.store.menu.toggle_btn"
-71. Select Store List,click,,"admin.store.submenu.store_list"
-72. Verify Add Store,verify,,"admin.store.list_page.header"
-73. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
-74. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-75. Click Doc Icon,click,,"admin.store.grid.doc_icon"
-76. Click Eye Icon,click,,"admin.store.grid.eye_view_icon"
-77. wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
-2. Click Delivery Services,click,,"admin.deliveryservice.menu"
-3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
-4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
-5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
-6. Click Stores,click,,"admin.store.menu.toggle_btn"
-7. Select Store List,click,,"admin.store.submenu.store_list"
-8. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
-9. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
-10. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-11. Click Product Icon,click,,"admin.store.products.grid_icon"
-12. Click Add Products,click,,"admin.store.products.add_btn"
-13. Open Product Category Dropdown,click,,"admin.store.products.category_dropdown"
-14. Select Grill Chicken,click,,"admin.store.products.category_option_grill"
-15. Enter Product Name,type,kfcProduct{randomAlpha}&gt;&gt; kfcProductName,"admin.store.products.name_input"
-16. Enter Product Amount,type,500,"admin.store.products.amount_input"
-17. Enter Product Description,type,KFC special grill chicken,"admin.store.products.description_textarea"
-18. Upload Product Image,uploadfile,"src/main/resources/test-data/grillchicken.jpg","admin.store.products.image.file"
-19. Open Product Category Dropdown,click,,"admin.store.products.status_dropdown"
-20. Select Activate,click,,"admin.store.products.status_option_active"
-21. Open Discount Type Dropdown,click,,"admin.store.products.discount_dropdown"
-22. Enter Discount Amount,type,50,"admin.store.products.discount_input"
-23. Click Save,click,,"admin.store.products.save_btn"
-24. Wait For Saved Succesfully,wait_until_visible,,"admin.store.products.toast_success"
-25. Wait For Store Products,wait_until_visible,,"admin.store.products.header"
-26. Filter Product List,type,{kfcProductName},"admin.store.products.name_filter"
-27. Click Back,click,,"admin.store.products.back_btn"
-28. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
-29. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-30. Click Wallet Icon,click,,"admin.store.wallet.grid_icon"
-31. Click Manage Transaction,click,,"admin.store.wallet.manage_transaction_btn"
-32. Enter Wallet Amount,type,1000,"admin.store.wallet.amount_input"
-33. Open Choose Option Dropdown,click,,"admin.store.wallet.option_dropdown"
-34. Select Add Money,click,,"admin.store.wallet.option_add"
-35. Click Submit,click,,"web.global.action.submit"
-36. Wait For Saved Succesfully,wait_until_visible,,"web.global.toast.success"
-37. Click Manage Transaction,click,,"admin.store.wallet.manage_transaction_btn"
-38. Enter Wallet Amount,type,200,"admin.store.wallet.amount_input"
-39. Open Choose Option Dropdown,click,,"admin.store.wallet.option_dropdown"
-40. Select Deduct Money,click,,"admin.store.wallet.option_deduct"
-41. Click Submit,click,,"web.global.action.submit"
-42. Wait For Saved Succesfully,wait_until_visible,,"web.global.toast.success"
-43. Click Back,click,,"admin.store.products.back_btn"
-44. Filter Store List,type,{storeName},"admin.store.grid.name_filter"
-45. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-46. Click Drivers Icon,click,,"admin.store.drivers.grid_icon"
-47. Click Add Private Driver,click,,"admin.store.drivers.add_private_btn"
-48. Enter Driver Name,type,kfcdriver_{timestamp} &gt;&gt; kfcdriverName,"admin.drivers.fullname.input"
-49. Enter Email,type,kfcdriver_{timestamp}@gmail.com,"admin.drivers.email.input"
-50. Enter Contact Number,type,{randomPhone},"admin.drivers.phone.input"
-51. Upload Profile Image,uploadfile,"src/main/resources/test-data/bikedriver.jpg","admin.drivers.profile_image.file"
-52. Select Male Gender,click,,"admin.drivers.male_gender.div"
-53. Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
-54. Select Scooter Option,click,,"admin.drivers.vehicle_option.scooter"
-55. Enter Model Year,type,2013,"admin.drivers.modelyear.input"
-56. Enter Vehicle Company,type,kfcBikeCompany{randomAlpha}&gt;&gt; kfcBikeCompanyName,"admin.drivers.companyname.input"
-57. Enter Plate No,type,KL-01-AB-1634,"admin.drivers.plateno.input"
-58. Enter Model Name,type,activa,"admin.drivers.modelname.input"
-59. Upload Vehicle Image,uploadfile,"src/main/resources/test-data/bike.jpg","admin.drivers.vehicle_image.file"
-60. Enter Vehicle Color,type,white,"admin.drivers.vehicle_color.input"
-61. Click Submit,click,,"web.global.action.submit"
-62. Wait For Driver Added,wait_until_visible,,"web.global.toast.success"
-63. Filter Driver List,type,{kfcdriverName},"admin.drivers.name_filter.input"
-64. Click Eye Icon,click,,"admin.store.grid.eye_view_icon"
-65. wait,1000,,</t>
-  </si>
-  <si>
-    <t>1. Click badge,click,,"admin.deliveryservice.badge.shield"
-2. Click Delivery Services,click,,"admin.deliveryservice.menu"
-3. Wait For Delivery Services,wait_until_visible,,"admin.deliveryservice.header"
-4. Click Home Icon Food Delivery,click,,"admin.store.food_delivery.home_icon"
-5. Wait For Food Delivery Summary,wait_until_visible,,"admin.store.food_delivery.summary_header"
-6. Click Stores,click,,"admin.store.menu.toggle_btn"
-7. Select Add Store,click,,"admin.store.submenu.add_store"
-8. Wait For Add Store,wait_until_visible,,"admin.store.add_page.header"
-9. Enter Store Name,type,bilal_{timestamp} &gt;&gt; hotelName,"admin.store.name.input"
-10. Open Delivery Radius Dropdown,click,,"admin.store.radius.dropdown"
-11. Select Twenty Five Kilometer,click,,"admin.store.radius.option_25km"
-12. Open Estimated Delivery Time,click,,"admin.store.eta.dropdown"
-13. Select Thirty Minute,click,,"admin.store.eta.option_30min"
-14. Enter Order Minimum Amount,type,300,"admin.store.min_amount.input"
-15. Enter Packaging Charges,type,50,"admin.store.packaging_charge.input"
-16. Enter Short Description,type,KFC is a global fast-food giant famous for its Original Recipe fried chicken,"admin.store.description.input"
-17. Upload Banner Image,uploadfile,"src/main/resources/test-data/kfcbanner.jpg","admin.store.banner.file"
-18. Open Driver Notification,click,,"admin.store.driver_notification.dropdown"
-19. Select Both Driver,click,,"admin.store.driver_notification.option_both"
-20. Click Checkbox Allow For Pickup,click,,"admin.store.allow_pickup.checkbox"
-21. Open Current Status Dropdown,click,,"admin.store.current_status.dropdown"
-22. Select Active,click,,"admin.store.current_status.option_active"
-23. Enter Store Address,type,KFC chennai,"admin.store.location.input"
-24. wait,3000,,
-25. Confirm Store Address,press_enter,,"admin.store.location.input"
-26. wait,3000,,
-27. Select First Option,arrow_down,,"admin.store.location.input"
-28. Confirm Option,press_enter,,"admin.store.location.input"
-29. wait,2000,,
-30. Click Storewise Comission Checkbox,click,,"admin.store.commission.checkbox"
-31. Enter Store Commision,type,25,"admin.store.commission_rate.input"
-32. Open Driver Notification,click,,"admin.store.offer_type.dropdown"
-33. Select Amount,click,,"admin.store.offer_type.option_amount"
-34. Enter Offer Amount,type,50,"admin.store.offer_amount.input"
-35. Enter Offer Min Amount,type,500,"admin.store.offer_min_amount.input"
-36. Enter Contact Person Full Name,type,bilalowner_{timestamp} &gt;&gt; hotelOwner,"admin.store.contact_name.input"
-37. Enter Email,type,bilal_{timestamp}@gmail.com&gt;&gt;storeEmail,"admin.store.email.input"
-38. Enter Contact Number,type,{randomPhone},"admin.store.phone.input"
-39. Upload Store Image,uploadfile,"src/main/resources/test-data/kfcstore.jpg","admin.store.profile.file"
-40. Enter Bank Name,type,federal,"admin.store.bank.name_input"
-41. Enter Bank Location,type,chennai,"admin.store.bank.location_input"
-42. Enter Account Number,type,123456789012,"admin.store.bank.account_input"
-43. Enter Accont Holder Name,type,{hotelOwner},"admin.store.bank.holder_input"
-44. Enter Payment Email Address,type,{storeEmail},"admin.store.bank.payment_email"
-45. Enter BIC Code,type,1234,"admin.store.bank.bic_input"
-46. Click Store Timing Checkbox,click,,"admin.store.timing.everyday_checkbox"
-47. Enter From Time,type,100000AM,"admin.store.timing.from_input"
-48. Enter To Time,type,100000PM,"admin.store.timing.to_input"
-49. Submit Add Store,click,,"web.global.action.submit"
-50. Wait For Success Message,wait_until_visible,,"web.global.toast.info"
-51. Click Stores,click,,"admin.store.menu.toggle_btn"
-52. Select Store List,click,,"admin.store.submenu.store_list"
-53. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
-54. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
-55. Click Stores,click,,"admin.store.menu.toggle_btn"
-56. Select Pending Documents Stores List,click,,"admin.store.submenu.pending_docs"
-57. Wait For Add Store,wait_until_visible,,"admin.store.pending_page.header"
-58. Filter Pending Document Store List,type,{hotelName},"admin.store.grid.name_filter"
-59. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-60. Click Doc Icon,click,,"admin.store.grid.doc_icon"
-61. Wait For Store Required Documents,wait_until_visible,,"admin.store.documents_page.header"
-62. Add Address Proof,click,,"admin.store.grid.edit_doc_icon"
-63. Upload Address Proof,uploadfile,"src/main/resources/test-data/addressproof.png","admin.store.doc.file_input"
-64. Enter Expiry Date,type,2026-12-12,"admin.store.doc.expiry_input"
-65. Click Submit,click,,"web.global.action.submit"
-66. Wait For Updated Succesfully,wait_until_visible,,"web.global.toast.updated"
-67. Click Approve Store,click,,"admin.store.grid.approve_doc_icon"
-68. Verify Updated Succesfully,verify,,"web.global.toast.updated"
-69. Click Back,click,,"admin.store.grid.back_btn"
-70. Click Stores,click,,"admin.store.menu.toggle_btn"
-71. Select Store List,click,,"admin.store.submenu.store_list"
-72. Wait For Add Store,wait_until_visible,,"admin.store.list_page.header"
-73. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
-74. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-75. Click Block Icon,click,,"admin.store.grid.block_icon"
-76. Click Block Yes,click,,"web.global.dialog.btn_confirm_yes"
-77. Click Stores,click,,"admin.store.menu.toggle_btn"
-78. Select Blocked Store,click,,"admin.store.submenu.blocked_stores"
-79. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
-80. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-81. Click unBlock Icon,click,,"admin.store.grid.unblock_icon"
-82. Click Stores,click,,"admin.store.menu.toggle_btn"
-83. Select Rejected Store,click,,"admin.store.submenu.rejected_stores"
-84. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
-85. Scroll Grid,tab,7,"admin.store.grid.name_filter"
-86. Click Approve Icon,click,,"admin.store.grid.approve_icon"
-87. Click Stores,click,,"admin.store.menu.toggle_btn"
-88. Select Store List,click,,"admin.store.submenu.store_list"
-89. Filter Store List,type,{hotelName},"admin.store.grid.name_filter"
-90. wait,3000,,
-91. Scroll Grid,tab,8,"admin.store.grid.name_filter"
-92. Click Doc Icon,click,,"admin.store.grid.document_icon"
-93. Click UnApprove Icon,click,,"admin.store.grid.unapprove_icon"
-94. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
-95. Rejection Reason,type,document insufficent,"web.global.dialog.textarea_reason"
-96. Click Reject Yes,click,,"web.global.dialog.btn_confirm_yes"
-97. wait,1000,,</t>
+117.wait for back button,wait,3000,
+118.Click Back, click, , "admin.store.grid.back_btn"
+119.Click Category, click, , "admin.deliveryservice.products.menu_category_btn"
+120.Click Add New Category, click, , "admin.deliveryservice.products.category.add_btn"
+121.Enter Category Name, type, curd{randomAlpha} &gt;&gt; MilkCategoryName, "admin.deliveryservice.products.category.name_input"
+122.Enter Category Name Arabic, type, رائب, "admin.deliveryservice.products.category.lang_arabic"
+123.Enter Category Name Tamil, type, தயிர், "admin.deliveryservice.products.category.lang_tamil"
+124.Enter Category Name Hindi, type, दही, "admin.deliveryservice.products.category.lang_hindi"
+125.Open Category status Dropdown, click, , "admin.deliveryservice.products.category.status_dropdown"
+126.Select Active, click, , "admin.deliveryservice.products.category.status_option_active"
+127.Upload Category Image, uploadfile, "src/main/resources/test-data/curd.jpeg", "admin.deliveryservice.image.file"
+128.wait, 2000, , ""
+129.Enter Slug Name, type, curd, "admin.deliveryservice.products.category.slug_input"
+130.Click Submit, click, , "web.global.action.submit"
+131.Verify Success Message, verify, , "web.global.toast.info"
+132.Filter Category Name, type, {MilkCategoryName}, "admin.deliveryservice.products.category.grid.filter_input"
+133.Click Stores, click, , "admin.store.menu.toggle_btn"
+134.Select Store List, click, , "admin.store.submenu.store_list"
+135.Filter Store List, type, {milkStore}, "admin.store.grid.name_filter"
+136.Scroll Grid, tab, 9, "admin.store.grid.name_filter"
+137.Click Product Icon, click, , "admin.store.products.grid_icon"
+138.Click Add Products, click, , "admin.store.products.add_btn"
+139.Open Product Category Dropdown, click, , "admin.store.products.category_dropdown"
+140.Select curd, click, , "admin.deliveryservice.products.category.option_dynamic"
+141.wait, 1000, ,""
+142.Click badge, click, , "admin.deliveryservice.badge.shield"
+143.Click Delivery Services, click, , "admin.deliveryservice.menu"
+144.Verify Delivery Services, verify, , "admin.deliveryservice.header"
+145.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+146.Click Edit Icon, click, , "admin.deliveryservice.grid.edit_icon"
+147.Open status Dropdown, click, , "admin.deliveryservice.status.dropdown"
+148.wait, 1000, , ""
+149.Select Deactivate, click, , "admin.deliveryservice.status.option_deactivate"
+150.Click Submit, click, , "web.global.action.submit"
+151.Filter Services List, type, {deliveryName}, "admin.deliveryservice.grid.filter_input"
+152.wait, 1000, ,</t>
   </si>
 </sst>
 </file>
@@ -3817,7 +3818,7 @@
         <v>28</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -3889,7 +3890,7 @@
         <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>111</v>
@@ -3961,7 +3962,7 @@
         <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>45</v>
@@ -4034,7 +4035,7 @@
         <v>57</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
9eth Commit:Set Date Keyword Updated
</commit_message>
<xml_diff>
--- a/we1_superAdmin_regression.xlsx
+++ b/we1_superAdmin_regression.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Hybrid_Framework\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDAA42DD-6314-4ABC-850C-0AA7A6F7CB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{512B79EF-7F04-4A2C-A84C-EFB163308031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="17" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SuperAdminLogin" sheetId="6" r:id="rId1"/>

</xml_diff>